<commit_message>
Actualización de BITACORA.xlsx desde Streamlit
</commit_message>
<xml_diff>
--- a/BITACORA.xlsx
+++ b/BITACORA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eycingenieria-my.sharepoint.com/personal/cristian_ramirez_eyc_com_co/Documents/Escritorio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EA987694-EA71-46D8-B76B-C3A33A0E2E8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{83B550CF-3404-402C-9A85-C89EF367B80D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F5425A24-549E-4FE1-A729-3B35E7CB95EF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9B58E14D-80FC-4389-A68E-EFFE3FA79470}"/>
   </bookViews>
   <sheets>
     <sheet name="2.01 Bitacora V10" sheetId="1" r:id="rId1"/>
@@ -5857,7 +5857,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A14CD2E1-D59E-4725-A57F-EDB3984F4403}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{452F15B9-CBB8-4BD6-BE48-A5CE4F394B5E}">
   <dimension ref="A1:AL515"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -48050,205 +48050,204 @@
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
-  <autoFilter ref="A1:AL515" xr:uid="{3EEE5335-66D3-4B3B-A1D2-2A445563FB56}"/>
   <hyperlinks>
-    <hyperlink ref="AL14" r:id="rId1" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzAxVG1GNlZrWlZiRkpQVkRKV2MxWllaRlZOVmtwUFdsVlZOVlpXV2xsaVJrSlRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{33B02BE4-F506-487A-91C2-E29FB4AE1049}"/>
-    <hyperlink ref="AL22" r:id="rId2" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkZKVVZsWlZiRkpQVkRKV2MxWllaRlZOUmtwVFZGVlZNV05XVGxWUmF6VlRVak5SZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{EB761618-A787-47A5-A2A2-0ECB5AE6665A}"/>
-    <hyperlink ref="AL25" r:id="rId3" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkZaVVJsWlZiRkpQVkRKV2MxWllaRlZOVmtwSFdsWlZOVlpXV2xWUmF6VlRVak5SZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{0810BC32-B59D-40A1-9FFF-497EE9B805B3}"/>
-    <hyperlink ref="AL26" r:id="rId4" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkZaVVJuaFZiRkpQVkRKV2MxWllaRlZOVmtwTFZGUkJNVTVzVmxsaFJUVlRVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{25BAD4BA-66B6-42F6-8B11-D3063AA8880F}"/>
-    <hyperlink ref="AL29" r:id="rId5" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkZaVVZuaFZiRkpQVkRKV2MxWllhRlZXYkVwRFZGZHplRkpXVGxWVGF6Vm9ZbGRSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{5FAB35BE-42A5-4E58-A351-B9676AFF3A71}"/>
-    <hyperlink ref="AL30" r:id="rId6" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkZaVVZUSlZiRkpQVkRKV2MxWllhRlZXYkVwRFZGWlZNVlpXVGxsYVJrSlhVak5SZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{0C4A2BEA-6808-4453-B700-483C3E8FE898}"/>
-    <hyperlink ref="AL32" r:id="rId7" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkdGNlJrWlZiRkpQVkRKV2MxWllhRlZXYkVwSFdsWlZlRTVzV2xsYVJUbFhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{FDCE1CB8-197A-46D0-8FAC-CA9BFDE09691}"/>
-    <hyperlink ref="AL33" r:id="rId8" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkdGNlJsWlZiRkpQVkRKV2MxWllaRlZOUmtwSFZGWlZNVkpXY0RaU2F6VnNZa2QzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{2EDB9012-1B69-420D-BC35-5322D296A455}"/>
-    <hyperlink ref="AL39" r:id="rId9" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkdGNmJFWlZiRkpQVkRKV2MxWllhRlZXVmtwaFZHdFZNV05XVmxWVmF6bG9ZbGRSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{62617166-8D03-45B0-8411-3E53FC67D43D}"/>
-    <hyperlink ref="AL40" r:id="rId10" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkdGNmJGWlZiRkpQVkRKV2MxWllhRlZXVmtwVFZHdFZlRTVzWkZsalJUVm9ZVEZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{FBFE99CA-EEF7-4562-BE32-9B6973A52B5F}"/>
-    <hyperlink ref="AL41" r:id="rId11" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGxKVVJrWlZiRkpQVkRKV2MxWllhRlZXVmtwWFdsWlZOVlpXWkZsalJUVlRVakEwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{F84D0F41-F6D5-4EA8-A080-E268D0DAB91A}"/>
-    <hyperlink ref="AL42" r:id="rId12" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGxKVVJuaFZiRkpQVkRKV2MxWllaRlZOVmtwUFZGWlZNV05XVmxWUmF6Vm9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{3D953E08-A2E4-4B0D-9142-95E38B2CE9F4}"/>
-    <hyperlink ref="AL44" r:id="rId13" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGxKVVZrWlZiRkpQVkRKV2MxWllaRlZOVmtwUFZGUkJOVlpXVmxsalJUbHNZa2QzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{B646D134-BC2A-4571-B69A-01512E038FE8}"/>
-    <hyperlink ref="AL45" r:id="rId14" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGxKVVZsWlZiRkpQVkRKV2MxWllaRlZOVmtwUFZHeFZOVkpXU2xWV2F6VlhVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{4F17CF7C-2988-44AC-AAF9-4F9A93A5463A}"/>
-    <hyperlink ref="AL46" r:id="rId15" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGxKVVZuaFZiRkpQVkRKV2MxWllaRlZOVmtwUFZGWlZlRTVzVWxsalJUbFRVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{3E58D647-32EA-4103-A468-523E175405B7}"/>
-    <hyperlink ref="AL47" r:id="rId16" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGxKVVZUSlZiRkpQVkRKV2MxWllaRlZOUmtwTFdsZHpNVTVzVGxsYVJUVlhVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{572FBFB6-19D7-4587-B4A7-55C9FAE73519}"/>
-    <hyperlink ref="AL50" r:id="rId17" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGxaVVJrWlZiRkpQVkRKV2MxWllaRlZOUmtwTFZGVlZOVkpXYkRaVGJFSlRVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{1E712A33-6E95-4CB4-BA7D-AB5D6F6A2E01}"/>
-    <hyperlink ref="AL52" r:id="rId18" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGxaVVJuaFZiRkpQVkRKV2MxWllhRlZXVmtwWFZGZHpNVTV0UmpaUmF6bHNZa1ZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{1D3A4FB9-32F8-4196-BBEB-343612AC863A}"/>
-    <hyperlink ref="AL53" r:id="rId19" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGxaVVJUSlZiRkpQVkRKV2MxWllhRlZXYkVwRFdsZHplRkpXUmxsaVJUVm9Za1ZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{4E5E9703-6519-4E31-A3DA-EFA712AE7C5C}"/>
-    <hyperlink ref="AL59" r:id="rId20" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVG1GNlJrWlZiRkpQVkRKV2MxWllhRlZXYkVwSFdsWlZNVkpXY0RaUmJFSlhVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{F7439828-D63F-41B5-A1D8-4E8A42E407DD}"/>
-    <hyperlink ref="AL60" r:id="rId21" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVG1GNlJsWlZiRkpQVkRKV2MxWllaRlZOUmtwWFZGWlZNV05XVmxWUmF6bFRVakEwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{800A094B-7DD3-4E33-A8E7-2541B278C883}"/>
-    <hyperlink ref="AL62" r:id="rId22" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVG1GNlJUSlZiRkpQVkRKV2MxWllaRlZOVmtwVFZGUkJNVkpXVWxWU2F6bG9ZVEJaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{D021ABAB-1CDB-4CB3-B34F-F76B386FCD1F}"/>
-    <hyperlink ref="AL63" r:id="rId23" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVG1GNlZrWlZiRkpQVkRKV2MxWllaRlZOVmtwVFdrUkJlR05XV2xWVmJFSlhVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{0E07C90B-CB47-42B0-9855-47857947580B}"/>
-    <hyperlink ref="AL65" r:id="rId24" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVG1GNlZuaFZiRkpQVkRKV2MxWllaRlZOVmtwTFZGVlZlRlpXWkZsaVJUbFRVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{E76CDD28-DEAF-4C2A-A5AD-EDDF68CDDC45}"/>
-    <hyperlink ref="AL67" r:id="rId25" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVG1GNmJFWlZiRkpQVkRKV2MxWllhRlZXYkVwRFZHdFZOVlpXUmxWVWF6VlRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{5C959BB6-1EE6-40BC-B59E-A341B2F26E5D}"/>
-    <hyperlink ref="AL68" r:id="rId26" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVG1GNmJGWlZiRkpQVkRKV2MxWllaRlZOVmtweFdsZHplRTVzVmxWVmF6bFhVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{EC6EAB67-2EBC-494A-B972-6ADDC45F1B3A}"/>
-    <hyperlink ref="AL69" r:id="rId27" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGsxRVJrWlZiRkpQVkRKV2MxWllhRlZXVmtwaFdsZHpNV05YUlhwalJUbFhVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{998FB17C-AFA2-4606-B280-7953DCFB1154}"/>
-    <hyperlink ref="AL70" r:id="rId28" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGsxRVJsWlZiRkpQVkRKV2MxWllaRlZOVmtwNVdsZHpNVkpXV2xsaFJUbFRVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{92DFE64D-08BB-4093-AAC7-687AE6A0565E}"/>
-    <hyperlink ref="AL73" r:id="rId29" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGsxRVZrWlZiRkpQVkRKV2MxWllhRlZXYkVwSFZHdFZNVlpXVWxWVmF6bG9ZWHBGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A1FC23B5-D0AE-4266-B0EC-B77B9AFDB4C1}"/>
-    <hyperlink ref="AL77" r:id="rId30" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGsxRWJFWlZiRkpQVkRKV2MxWllaRlZOVmtwTFZGZHpOVlpXU2xsalJUbFRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{D3E5A685-9F7A-4389-9AB2-C102DEC945C6}"/>
-    <hyperlink ref="AL82" r:id="rId31" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVDFKVVJUSlZiRkpQVkRKV2MxWllhRlZXVmtwSFdsZHpOVlpXVmxsalJUVnNZWHBGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{141EB394-A5CE-47AB-9008-184E372B35E1}"/>
-    <hyperlink ref="AL83" r:id="rId32" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVDFKVVZrWlZiRkpQVkRKV2MxWllaRlZOUmtwaFZGZHpOVkpXVmxsYVJUVlhVak5SZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{02D52B90-45D3-4390-927C-256FEC44A9E6}"/>
-    <hyperlink ref="AL87" r:id="rId33" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVDFaVVJsWlZiRkpQVkRKV2MxWllhRlZXVmtweFdsWlZlR05XVGxsalJUbFRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{991DA42E-982F-4A47-B7C5-D34718DE668F}"/>
-    <hyperlink ref="AL88" r:id="rId34" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVDFaVVJuaFZiRkpQVkRKV2MxWllaRlZOVmtwMVZGVlZNV05XVWxsalJUVlRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{720EA7B3-693C-40AE-A68E-4A39FA2D19DC}"/>
-    <hyperlink ref="AL89" r:id="rId35" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVDFaVVJUSlZiRkpQVkRKV2MxWllaRlZOVmtwUFdsVlZlRTVzVWxWVGJFSlRVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{2020E683-5750-4CD1-B632-135F28869106}"/>
-    <hyperlink ref="AL90" r:id="rId36" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVDFaVVZrWlZiRkpQVkRKV2MxWllaRlZOUmtwaFZGWlZNVlpXWkZWVGF6bG9ZVEZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{3A782AEE-6FB0-477D-90FF-98F618983D0F}"/>
-    <hyperlink ref="AL98" r:id="rId37" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYTAxRVZrWlZiRkpQVkRKV2MxWllaRlZOUmtwSFZHeFZlR05XY0RaV2F6VlRVak5SZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{27772D85-D82A-4CF8-B1DF-C4F46312DCC2}"/>
-    <hyperlink ref="AL103" r:id="rId38" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYTAxRWJGWlZiRkpQVkRKV2MxWllaRlZOUmtwSFZHeFZlRkpXWkZWVGF6bHNZbGhSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{BFE8331B-0675-4992-BA70-956659C88E78}"/>
-    <hyperlink ref="AL104" r:id="rId39" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZKVVJrWlZiRkpQVkRKV2MxWllhRlZXVmtwTFZGWlZlRkpXVWxWVmF6VnNZVEJaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A7F3EA48-779C-4150-B641-7E10B7D541DE}"/>
-    <hyperlink ref="AL107" r:id="rId40" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZKVVJUSlZiRkpQVkRKV2MxWllhRlZXVmtwWFZGZHpNVTVzWkZWV2F6bFRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{84358B77-CCF9-4388-8F51-85FD101F80E1}"/>
-    <hyperlink ref="AL108" r:id="rId41" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZKVVZrWlZiRkpQVkRKV2MxWllaRlZOUmtwRFdsZHpNVTVzUmxsYVJUbHNZVEZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{64D24858-40A3-4427-84C5-1B5BF0510B42}"/>
-    <hyperlink ref="AL109" r:id="rId42" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZKVVZsWlZiRkpQVkRKV2MxWllaRlZOUmtwSFdrUkJlRlpXU2xWVmF6bFhVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{7112E70C-7248-4EC8-84CE-7E3D2A1F4967}"/>
-    <hyperlink ref="AL110" r:id="rId43" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZKVVZuaFZiRkpQVkRKV2MxWllhRlZXYkVwTFdrUkJlRlpXUmxsaFJUbFhVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{35CA87FC-83D2-44DF-AFD9-62E63C48FFAB}"/>
-    <hyperlink ref="AL111" r:id="rId44" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZKVVZUSlZiRkpQVkRKV2MxWllaRlZpYmtKeFZGZHpNVlpXWkZsalJUVm9Za2QzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{731CAFA4-AF23-420D-BAFF-2CA0DF6747BD}"/>
-    <hyperlink ref="AL112" r:id="rId45" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZKVWJFWlZiRkpQVkRKV2MxWllaRlZpYmtKMVZGVlZNVTVzYkRaU2F6VlRVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{34877C06-BC68-438D-9DE9-F5B43A7BB3C8}"/>
-    <hyperlink ref="AL115" r:id="rId46" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZaVVJsWlZiRkpQVkRKV2MxWllaRlZOVmtwVFdsVlZlRkpXUmxsaFJUbFhVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A39E550C-6E14-4019-9088-908BB0470210}"/>
-    <hyperlink ref="AL119" r:id="rId47" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZaVVZsWlZiRkpQVkRKV2MxWllhRlZXVmtwUFZGUkJOVkpXYjNwalJUbG9ZbGhSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{D3A94EBE-B70B-4665-A5FF-3CB0B74FC93E}"/>
-    <hyperlink ref="AL120" r:id="rId48" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZaVVZuaFZiRkpQVkRKV2MxWllaRlZOVmtwVFdsVlZNVlpXVmxsaVJUbFRVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{B39AAB58-F22E-4247-A190-90AA542A77E4}"/>
-    <hyperlink ref="AL121" r:id="rId49" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZaVVZUSlZiRkpQVkRKV2MxWllaRlZOVmtwNVZGVlZlRlpXVWxWVmF6Vm9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{63035E67-BD28-41CA-9890-779557DB949F}"/>
-    <hyperlink ref="AL122" r:id="rId50" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZaVWJFWlZiRkpQVkRKV2MxWllhRlZXVmtwNVZGUkJOVlpXUmxWVGF6bHNZa2QzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{66365AB7-C39C-4499-9059-ABFE4B1B56E5}"/>
-    <hyperlink ref="AL123" r:id="rId51" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZaVWJGWlZiRkpQVkRKV2MxWllaRlZOVmtwUFZGZHpNVkpXYjNwYVJUbFRVakEwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{BFF7300B-3355-424F-ACF9-FEFF06BBAE6B}"/>
-    <hyperlink ref="AL125" r:id="rId52" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkdGNlJsWlZiRkpQVkRKV2MxWllaRlZOUmtwSFZGUkJlR05XVWxsaFJUVm9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{39F70EC0-E279-43B5-AA6F-8C136490DCDC}"/>
-    <hyperlink ref="AL126" r:id="rId53" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkdGNlJuaFZiRkpQVkRKV2MxWllaRlZOVmtwUFZGUkJOVlpXVWxsaFJUbHNZbGRSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{36E8128E-98F2-4F13-BB3F-2A4CC8B03BDC}"/>
-    <hyperlink ref="AL127" r:id="rId54" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkdGNlJUSlZiRkpQVkRKV2MxWllaRlZOUmtwTFZHeFZOVkpXUmxsYVJUVlRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{C3C332FC-8817-42EB-9ABF-049D8CAAEADF}"/>
-    <hyperlink ref="AL128" r:id="rId55" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkdGNlZrWlZiRkpQVkRKV2MxWllaRlZpYmtKNVdsZHplRTVzV2xWVmJFSlRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{3CE6D38D-1056-4284-8001-2323FB6701C4}"/>
-    <hyperlink ref="AL129" r:id="rId56" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkdGNlZsWlZiRkpQVkRKV2MxWllaRlZOUmtwRFdsZHpNVkpXYTNwalJUbFhVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{77747356-FF53-460F-8113-90194FFF2CFC}"/>
-    <hyperlink ref="AL131" r:id="rId57" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkdGNlZUSlZiRkpQVkRKV2MxWllhRlZXVmtwMVZHeFZlR05XVmxWVWJFSlRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{8591474E-A25E-4C64-B197-F654FD086C6A}"/>
-    <hyperlink ref="AL132" r:id="rId58" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkdGNmJFWlZiRkpQVkRKV2MxWllhRlZXVmtwMVZGWlZlRTVzV2xWVWJFSlhVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{C8768FFB-FFD1-45C2-9314-D689E108C664}"/>
-    <hyperlink ref="AL133" r:id="rId59" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkdGNmJGWlZiRkpQVkRKV2MxWllhRlZXVmtwMVdrUkJOVkpXVWxsYVJUVm9ZbGhSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{E3E7E892-2650-476E-BAA5-22C535D4A021}"/>
-    <hyperlink ref="AL134" r:id="rId60" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxKVVJrWlZiRkpQVkRKV2MxWllhRlZXVmtwaFdsZHplR05XYkRaU2F6VlRVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{98C20155-8AB9-438D-972C-C09180C0FEB8}"/>
-    <hyperlink ref="AL136" r:id="rId61" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxKVVJuaFZiRkpQVkRKV2MxWllaRlZOUmtwRFZHdFZlR05YUmpaUmF6bFhVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{6AD5BC00-EDC6-476A-8733-C33A3F2D00A0}"/>
-    <hyperlink ref="AL138" r:id="rId62" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxKVVZsWlZiRkpQVkRKV2MxWllaRlZOVmtwRFZGWlZNVkpXU2xWV2F6bFRVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{AAA40C2F-50E4-4665-8CBA-0ACCCB6D1F9C}"/>
-    <hyperlink ref="AL139" r:id="rId63" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxKVVZuaFZiRkpQVkRKV2MxWllaRlZOUmtweFdsVlZlRlpXVmxWVWF6bHNZbGhSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{354BCFD6-0D26-478F-845E-9B2CF482804F}"/>
-    <hyperlink ref="AL140" r:id="rId64" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxKVVZUSlZiRkpQVkRKV2MxWllaRlZOUmtweFdsZHpOVlpXU2xsalJUbFRVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{7ED35994-7B82-4AD8-BE56-33F34CE54CD0}"/>
-    <hyperlink ref="AL142" r:id="rId65" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxKVWJGWlZiRkpQVkRKV2MxWllaRlZOVmtwWFdrUkJOVkpXV2xWVWF6bFhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{EE5D1C00-30FE-4AF0-8B8D-C1D004F36584}"/>
-    <hyperlink ref="AL144" r:id="rId66" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxaVVJsWlZiRkpQVkRKV2MxWllaRlZOVmtwTFdsVlZOVlpYUmpaVGF6bFhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{6228E79B-7951-456F-AFA3-1B72363C083B}"/>
-    <hyperlink ref="AL146" r:id="rId67" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxaVVJUSlZiRkpQVkRKV2MxWllhRlZXVmtweFdsZHpNV05XVmxsaVJrSlRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{9ACD0DCC-4585-4CF3-A6D4-175EA7AEDAF6}"/>
-    <hyperlink ref="AL149" r:id="rId68" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxaVVZuaFZiRkpQVkRKV2MxWllaRlZOUmtwUFZGWlZNVkpXYkRaU2F6VnNZa2QzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{4975175C-4D58-4041-A1F1-848AE621CC26}"/>
-    <hyperlink ref="AL151" r:id="rId69" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxaVWJFWlZiRkpQVkRKV2MxWllaRlZOUmtwaFdrUkJOVlpXVmxsaFJUbG9Za1paZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{0305E0B0-6725-47E1-977B-68DACBB4A185}"/>
-    <hyperlink ref="AL153" r:id="rId70" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVG1GNlJrWlZiRkpQVkRKV2MxWllaRlZOUmtwTFZGWlZlR05XVWxsalJUbG9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{F3735334-C8ED-4A7D-BE35-BF901CEDC655}"/>
-    <hyperlink ref="AL155" r:id="rId71" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVG1GNlJuaFZiRkpQVkRKV2MxWllhRlZXVmtwTFZHeFZlRkpXUmxsaVJUbG9ZWHBGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{3156F6F3-135A-4792-AE6C-D13524F38571}"/>
-    <hyperlink ref="AL160" r:id="rId72" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVG1GNmJFWlZiRkpQVkRKV2MxWllaRlZOVmtwSFdrUkJlR05XVmxWVGF6VlhVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{BD2B2CE2-58C5-43E9-9558-073E5E988E59}"/>
-    <hyperlink ref="AL161" r:id="rId73" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVG1GNmJGWlZiRkpQVkRKV2MxWllhRlZXVmtwVFZHeFZNVkpXU2xsaVJUVlRVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{B608A34C-1E15-433B-BF86-4C092404E22B}"/>
-    <hyperlink ref="AL163" r:id="rId74" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGsxRVJsWlZiRkpQVkRKV2MxWllhRlZXVmtwTFdsZHpNVTVzVGxWVmF6VlhVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A6C8F117-708B-4ABE-8D43-BC9079807BCD}"/>
-    <hyperlink ref="AL166" r:id="rId75" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGsxRVZrWlZiRkpQVkRKV2MxWllhRlZXVmtwVFdrUkJNVlpXYjNwalJUbFhVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{E3DAF800-3849-44EF-BCE5-6CD52B1E7736}"/>
-    <hyperlink ref="AL168" r:id="rId76" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGsxRVZuaFZiRkpQVkRKV2MxWllaRlZOVmtwUFdsVlZlRkpXVmxsalJUbFhVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{C45336AF-E43E-4560-A400-093D7ECC5583}"/>
-    <hyperlink ref="AL171" r:id="rId77" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGsxRWJGWlZiRkpQVkRKV2MxWllaRlZOVmtwTFdsZHpNV05XY0RaUmF6Vm9ZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{42A7135B-7643-4C08-8B7B-8EA716FE84C9}"/>
-    <hyperlink ref="AL172" r:id="rId78" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVDFKVVJrWlZiRkpQVkRKV2MxWllhRlZXVmtwVFZGUkJlRlpXV2xWVGF6bFhVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{771B2D26-CC39-46BB-AA4E-001ECD41CF8E}"/>
-    <hyperlink ref="AL176" r:id="rId79" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVDFKVVZrWlZiRkpQVkRKV2MxWllhRlZXVmtwMVZHeFZNVTVzYTNwaFJUbFhVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{5B591698-8866-4589-B32A-3323BE412F08}"/>
-    <hyperlink ref="AL177" r:id="rId80" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVDFKVVZsWlZiRkpQVkRKV2MxWllaRlZOVmtwWFZGVlZlRlpXV2xsYVJUbFhVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A297580F-7EEC-4648-9CBD-EB94ADAACBB2}"/>
-    <hyperlink ref="AL178" r:id="rId81" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVDFKVVZuaFZiRkpQVkRKV2MxWllaRlZOUmtwMVZGVlZOVkpXYTNwaVJUVlhVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{0F6757F0-F633-49CE-8814-E5F45BCDD496}"/>
-    <hyperlink ref="AL179" r:id="rId82" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVDFKVVZUSlZiRkpQVkRKV2MxWllaRlZOUmtwNVdsZHpOVlpXYkRaVmF6bHNZbGRSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{4BC107AF-E08D-41B1-A95F-DB68FE9F33F8}"/>
-    <hyperlink ref="AL182" r:id="rId83" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVDFaVVJrWlZiRkpQVkRKV2MxWllaRlZpYmtKMVZGVlZlRkpXYkRaVmF6bFhVakEwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{573BA32D-C70C-4FD8-991B-FB6A022BED54}"/>
-    <hyperlink ref="AL183" r:id="rId84" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVDFaVVJsWlZiRkpQVkRKV2MxWllhRlZXVmtwMVdsZHpOVkpXUmxWVmF6VlhVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{72BC9113-94FA-48DF-8EBF-C9A5EBBFEB0E}"/>
-    <hyperlink ref="AL186" r:id="rId85" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVDFaVVZrWlZiRkpQVkRKV2MxWllaRlZOVmtwaFdsVlZlRTVzVGxsaFJUVlRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{9F40AA84-4B92-41B6-B8D3-B1315C506101}"/>
-    <hyperlink ref="AL191" r:id="rId86" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYTAxRVJrWlZiRkpQVkRKV2MxWllaRlZOUmtwaFZGVlZOVkpXYTNwYVJUbG9ZbGhSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{6A822038-2D4A-4B7F-8ECB-2B244403298C}"/>
-    <hyperlink ref="AL192" r:id="rId87" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYTAxRVJsWlZiRkpQVkRKV2MxWllhRlZXYkVwSFdsZHplRkpYUmpaUmJFSlRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{606D22C5-573F-4617-A2C7-EFE291FF5C22}"/>
-    <hyperlink ref="AL193" r:id="rId88" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYTAxRVJuaFZiRkpQVkRKV2MxWllaRlZOVmtwRFdsZHpNV05YUlhwYVJUbG9Za2QzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{869B7F59-C362-4CF5-9EDF-7BD9B73F1DC1}"/>
-    <hyperlink ref="AL196" r:id="rId89" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYTAxRVZsWlZiRkpQVkRKV2MxWllaRlZOUmtwNVZGZHpOVkpXVmxsaFJUVnNZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{20C864CE-0F5F-4D63-8226-A0024ECDBBB7}"/>
-    <hyperlink ref="AL197" r:id="rId90" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYTAxRVZuaFZiRkpQVkRKV2MxWllaRlZOUmtwRFZGVlZNVlpXU2xWV2F6bG9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{7B2B698E-21F3-4995-93D6-38A8317DE16B}"/>
-    <hyperlink ref="AL199" r:id="rId91" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYTAxRWJFWlZiRkpQVkRKV2MxWllaRlZOVmtwSFZGUkJOVlpXU2xsalJUbFhVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{8DDE2732-EA23-4E95-958C-9098CC7EAAB1}"/>
-    <hyperlink ref="AL201" r:id="rId92" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYkZKVVJrWlZiRkpQVkRKV2MxWllhRlZXVmtwVFZGZHplRlpXVGxWUmJFSlhVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{B0C4AB84-F94F-4A90-A437-36B622E3348A}"/>
-    <hyperlink ref="AL203" r:id="rId93" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYkZKVVJuaFZiRkpQVkRKV2MxWllaRlZOUmtwNVdsVlZNVlpXVWxWV2F6VlhVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{37EB19B8-39A6-4BD3-9F35-8237DDEFFA85}"/>
-    <hyperlink ref="AL206" r:id="rId94" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYkZKVVZuaFZiRkpQVkRKV2MxWllhRlZXYkVwRFdsWlZlRlpXU2xsalJUbFhVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{5D8C14F5-D936-456E-AE62-F20E6B617644}"/>
-    <hyperlink ref="AL211" r:id="rId95" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYkZaVVJuaFZiRkpQVkRKV2MxWllaRlZOUmtwWFZGWlZlRlpXWkZsaFJUbG9ZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{602AF86C-0981-4B4D-9476-947F6B4FF26C}"/>
-    <hyperlink ref="AL212" r:id="rId96" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYkZaVVZrWlZiRkpQVkRKV2MxWllaRlZOUmtwRFdsVlZlR05YUmpaVWJFSlhVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{C86DAD52-A544-4F17-8536-EA662A4A5F6D}"/>
-    <hyperlink ref="AL221" r:id="rId97" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYkdGNlZsWlZiRkpQVkRKV2MxWllaRlZOUmtwSFZGVlZNV05XWkZsYVJUbFhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{42722779-0E5C-4CB2-A0DD-A28B09759D7B}"/>
-    <hyperlink ref="AL226" r:id="rId98" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhVGxKVVZrWlZiRkpQVkRKV2MxWllaRlZOUmtwMVZGVlZOVlpXUmxWU2F6VnNZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{BFCF9870-AC05-4C81-96B9-453AA4BA1463}"/>
-    <hyperlink ref="AL227" r:id="rId99" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhVGxKVVZsWlZiRkpQVkRKV2MxWllaRlZOVmtwWFdsWlZNVkpXVmxsaVJUbHNZVEJaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{C6F12071-5B7A-49FC-87B1-99BA48E99C02}"/>
-    <hyperlink ref="AL228" r:id="rId100" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhVGxKVVZuaFZiRkpQVkRKV2MxWllaRlZOVmtwVFdrUkJNVkpYUmpaU2F6bHNZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{115B60E5-5150-4FCF-B64B-2971811CAA77}"/>
-    <hyperlink ref="AL232" r:id="rId101" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYTAxRVJuaFZiRkpQVkRKV2MxWllaRlZOUmtwWFZGZHplRTVzWkZWUmF6bFhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{4DDB205D-5E80-4DAC-9869-890A5E7DC11D}"/>
-    <hyperlink ref="AL233" r:id="rId102" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYTAxRVJUSlZiRkpQVkRKV2MxWllaRlZOUmtwaFZGUkJlRTVzVWxsalJUVlhVak5SZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{5A4D3160-7FE8-479D-84DB-5BA174228C40}"/>
-    <hyperlink ref="AL234" r:id="rId103" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYTAxRVZrWlZiRkpQVkRKV2MxWllaRlZOUmtwMVZHdFZlRkpXWkZWVGJFSlhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{8DC82E76-3D1F-4188-BED3-17D96218D62E}"/>
-    <hyperlink ref="AL235" r:id="rId104" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYTAxRVZsWlZiRkpQVkRKV2MxWllaRlZOUmtwaFdrUkJlRkpXVmxsYVJUVnNZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{6D9D2E8E-8107-43E8-9EF8-9E59BBD22F91}"/>
-    <hyperlink ref="AL236" r:id="rId105" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYTAxRVZUSlZiRkpQVkRKV2MxWllaRlZOVmtwMVZGVlZNVlpXVWxWVWF6bFhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{BCC8D2D6-C2C4-4148-B295-C9E461059F16}"/>
-    <hyperlink ref="AL237" r:id="rId106" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYTAxRWJFWlZiRkpQVkRKV2MxWllhRlZXVmtwVFdsVlZNVTVzU2xsaFJUVlRVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{380FFA42-0BC3-4598-AE4C-78B8C5683FD8}"/>
-    <hyperlink ref="AL238" r:id="rId107" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYTAxRWJGWlZiRkpQVkRKV2MxWllhRlZXVmtweFdsVlZNVkpXVWxWUmF6bHNZbGhSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{8A24726E-6342-496E-B92E-836FFC8226AA}"/>
-    <hyperlink ref="AL239" r:id="rId108" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYkZKVVJrWlZiRkpQVkRKV2MxWllaRlZOUmtwUFZGZHplRlpXU2xWVGF6bG9ZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{9FED67E8-C280-438A-B3E3-1502AAD58814}"/>
-    <hyperlink ref="AL243" r:id="rId109" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYkZKVVZrWlZiRkpQVkRKV2MxWllhRlZXVmtwMVdsWlZNV05XVWxWV2F6Vm9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{0CD099C5-B868-4278-977E-5D2E467EC02C}"/>
-    <hyperlink ref="AL247" r:id="rId110" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYkZaVVJUSlZiRkpQVkRKV2MxWllhRlZXVmtwVFZGZHpOVkpXVmxWVGF6Vm9Za1paZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A0BCBCF4-5310-4B23-A38C-83568C20B9DA}"/>
-    <hyperlink ref="AL248" r:id="rId111" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYkZaVVZuaFZiRkpQVkRKV2MxWllhRlZXVmtwMVdsWlZlRTVzY0RaVWF6bFRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{6C49DCE8-41BF-4C14-A2BE-61903A08EAE3}"/>
-    <hyperlink ref="AL249" r:id="rId112" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYkdGNlZsWlZiRkpQVkRKV2MxWllaRlZOVmtwSFZGWlZlR05XVGxWVGF6bHNZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{E2D3C4B9-C47E-4A0D-91D3-E14FB3A0E439}"/>
-    <hyperlink ref="AL250" r:id="rId113" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYkdGNmJFWlZiRkpQVkRKV2MxWllhRlZXVmtwTFZGZHpOVlpXV2xsaFJUbFRVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A2C9874B-50AC-406D-8D5F-083132AB0D91}"/>
-    <hyperlink ref="AL251" r:id="rId114" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYkdGNmJGWlZiRkpQVkRKV2MxWllaRlZOVmtwUFZGWlZNVlpXUmxWVmF6bFhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{33012BD0-A553-452A-8F83-1A38002502FC}"/>
-    <hyperlink ref="AL252" r:id="rId115" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxVGxKVVJsWlZiRkpQVkRKV2MxWllaRlZOUmtweFdsVlZNVlpXVmxWVWF6bG9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{59ABEF5E-D7D7-46C3-B95C-0E86E2FE06C5}"/>
-    <hyperlink ref="AL254" r:id="rId116" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxVGxKVVZrWlZiRkpQVkRKV2MxWllhRlZXVmtwMVdsVlZOVkpYUmpaVmF6bFhVak5SZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{E479EDE1-90EA-42DE-81AD-9529CFF8F0B3}"/>
-    <hyperlink ref="AL255" r:id="rId117" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxVGxKVVZsWlZiRkpQVkRKV2MxWllhRlZXVmtwNVZGZHpOVlpYUlhwaFJUbG9ZWHBGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{7D473499-1608-4BB1-B545-8CEA29477205}"/>
-    <hyperlink ref="AL256" r:id="rId118" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxVGxKVVZuaFZiRkpQVkRKV2MxWllhRlZXVmtwMVZGZHpNVkpXYjNwYVJUbFRVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{BA5BE7C1-CA5C-45E9-8ADC-EA42B15F3686}"/>
-    <hyperlink ref="AL257" r:id="rId119" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxVGxKVVZUSlZiRkpQVkRKV2MxWllhRlZXVmtwNVdsWlZlRlpXY0RaU2F6bG9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{118E2B5F-2D9D-4219-BD2B-2D109A22C96D}"/>
-    <hyperlink ref="AL261" r:id="rId120" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLYkZaVVZsWlZiRkpQVkRKV2MxWllaRlZOUmtwNVZHdFZOVlpYUmpaU2F6bFRVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{8CE14E63-5765-4ED1-85ED-1697783BC620}"/>
-    <hyperlink ref="AL263" r:id="rId121" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLYkZaVWJGWlZiRkpQVkRKV2MxWllaRlZOVmtwMVdrUkJlRTVzV2xWU2JFSlRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{E198F40F-4AFD-424B-BD83-7EA935A55D1E}"/>
-    <hyperlink ref="AL266" r:id="rId122" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLYkdGNlZuaFZiRkpQVkRKV2MxWllhRlZXYkVwRFZGWlZOVkpXU2xWV2F6bHNZa1ZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{F42A881F-4F0E-42D0-B522-3C07B606899A}"/>
-    <hyperlink ref="AL268" r:id="rId123" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLYkdGNmJFWlZiRkpQVkRKV2MxWllaRlZOVmtwWFdsVlZNVkpXVWxWV2F6Vm9ZWHBGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{D2E45ADB-3D99-4EBE-B949-96166C990682}"/>
-    <hyperlink ref="AL271" r:id="rId124" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGxKVVJsWlZiRkpQVkRKV2MxWllhRlZXVmtwWFdrUkJOVlpXYTNwaVJUVlhVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{B7B2B388-1213-42B3-904B-DC7ED7A2C225}"/>
-    <hyperlink ref="AL275" r:id="rId125" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGxKVVZuaFZiRkpQVkRKV2MxWllhRlZXVmtwTFZHeFZlRlpXVGxsalJUVlRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{4E769D3E-E0CC-4953-AF19-AA2C8F7F31AD}"/>
-    <hyperlink ref="AL277" r:id="rId126" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGxKVWJFWlZiRkpQVkRKV2MxWllhRlZXVmtweFZGWlZlRlpXY0RaVWF6VnNZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{538F7867-1124-4E73-BF33-406C942D0D14}"/>
-    <hyperlink ref="AL278" r:id="rId127" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGxKVWJGWlZiRkpQVkRKV2MxWllaRlZOUmtwUFZGVlZNVTVzVWxWUmF6Vm9Za1paZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{771FD09E-A433-47ED-A911-624916758128}"/>
-    <hyperlink ref="AL281" r:id="rId128" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGxaVVJUSlZiRkpQVkRKV2MxWllaRlZOUmtwRFZGUkJNVTV0UmpaV2F6bFRVakEwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{9A18AC04-210F-4D15-A483-E7B6FB90556B}"/>
-    <hyperlink ref="AL286" r:id="rId129" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGxaVWJFWlZiRkpQVkRKV2MxWllhRlZXVmtwNVdsVlZlRTVzWkZWV2F6Vm9ZbGRSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{8C2971DD-ACC0-49C6-B08E-0611DCC2BE17}"/>
-    <hyperlink ref="AL287" r:id="rId130" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGxaVWJGWlZiRkpQVkRKV2MxWllhRlZXVmtwVFZHdFZlRkpXWkZsYVJrSlRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{C4029854-E658-401D-BCD5-C003E64F0BFE}"/>
-    <hyperlink ref="AL290" r:id="rId131" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVG1GNlJUSlZiRkpQVkRKV2MxWllaRlZOUmtwSFdsVlZOVlpXUmxWUmF6VnNZbGhSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{0D0A9F31-41E3-42D4-A33E-46AE1F4EC909}"/>
-    <hyperlink ref="AL291" r:id="rId132" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVG1GNlZrWlZiRkpQVkRKV2MxWllaRlZOVmtwMVdsVlZlRlpXU2xWUmF6VlRVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{508D72B0-FE38-4FF9-8CEF-73935ABCF6C1}"/>
-    <hyperlink ref="AL292" r:id="rId133" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVG1GNlZsWlZiRkpQVkRKV2MxWllaRlZOVmtwVFZGVlZlRlpXY0RaVmF6VlRVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{2C7FE904-D276-47EC-8553-6D65D44EB5CF}"/>
-    <hyperlink ref="AL293" r:id="rId134" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVG1GNlZuaFZiRkpQVkRKV2MxWllaRlZOUmtwWFdsVlZNVlpXVmxWVmF6bG9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{916C796F-128C-496A-B43D-A02C223A001F}"/>
-    <hyperlink ref="AL295" r:id="rId135" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVG1GNmJFWlZiRkpQVkRKV2MxWllaRlZOUmtwSFZGZHpOVlpXUmxsalJrSlhVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{62BD5853-D495-4CDF-AC70-0C189FC1845F}"/>
-    <hyperlink ref="AL297" r:id="rId136" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGsxRVJrWlZiRkpQVkRKV2MxWllhRlZXVmtwUFdsVlZNVkpXYTNwalJUVnNZa1paZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{4A922A4D-922B-4066-B144-87DCD4B059B7}"/>
-    <hyperlink ref="AL299" r:id="rId137" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGsxRVJuaFZiRkpQVkRKV2MxWllhRlZXVmtwWFZGVlZNVTV0UlhwaVJUbFRVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{72FC73C9-36D1-4BA7-BDD7-54D26C9F6A32}"/>
-    <hyperlink ref="AL300" r:id="rId138" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGsxRVJUSlZiRkpQVkRKV2MxWllaRlZOVmtwWFdsZHpNVlpXYTNwalJrSlhVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{59E56EB4-2974-4F1E-90A9-FA01BF4C5898}"/>
-    <hyperlink ref="AL302" r:id="rId139" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGsxRVZuaFZiRkpQVkRKV2MxWllaRlZOUmtwWFdrUkJNVkpYUmpaU2F6VlRVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{E45ED0BD-D1BF-4A10-BEB8-3B16F9267A69}"/>
-    <hyperlink ref="AL304" r:id="rId140" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGsxRWJFWlZiRkpQVkRKV2MxWllaRlZOVmtwUFdsZHplRkpXYjNwYVJUbHNZbGRSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{9D6886F2-DDD8-4473-955F-A8696560E80B}"/>
-    <hyperlink ref="AL305" r:id="rId141" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGsxRWJGWlZiRkpQVkRKV2MxWllaRlZOVmtwRFdrUkJlRlpXYjNwYVJUVlRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{23DE19A4-0D5F-46AB-9F56-1AA678C0EDCF}"/>
-    <hyperlink ref="AL306" r:id="rId142" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFKVVJrWlZiRkpQVkRKV2MxWllaRlZOVmtwWFZHdFZlRlpXV2xsalJUbG9ZbGhSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{38E23B8E-E88F-41F8-8333-3B512B3B7BB1}"/>
-    <hyperlink ref="AL307" r:id="rId143" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFKVVJsWlZiRkpQVkRKV2MxWllaRlZOVmtwRFZHeFZOVlpXVGxWU2F6bG9ZbGRSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A35B160D-BB83-4A62-883E-E4D2E58EE9E0}"/>
-    <hyperlink ref="AL308" r:id="rId144" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFKVVJuaFZiRkpQVkRKV2MxWllhRlZXVmtwWFZHdFZNVkpXU2xsYVJUbG9ZbGRSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{9C680734-455B-404E-9CE6-B65CE0F1266F}"/>
-    <hyperlink ref="AL309" r:id="rId145" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFKVVJUSlZiRkpQVkRKV2MxWllaRlZOVmtwSFZHdFZlRlpXUmxsaFJUbFRVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{201BB15A-D79D-4A07-9C35-3CFAC7C5E9EC}"/>
-    <hyperlink ref="AL312" r:id="rId146" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFKVVZuaFZiRkpQVkRKV2MxWllaRlZOVmtwUFdsVlZlR05XVmxsaVJrSlhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{83A54ADE-B8FF-431A-9C97-D04C7B3CBDFE}"/>
-    <hyperlink ref="AL313" r:id="rId147" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFKVVZUSlZiRkpQVkRKV2MxWllhRlZXVmtweFdsWlZNVkpXYkRaVWJFSlRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{7B9BAF5C-6592-4B74-8DC4-282457E9E10C}"/>
-    <hyperlink ref="AL320" r:id="rId148" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFaVVZrWlZiRkpQVkRKV2MxWllaRlZpYmtKNVZGWlZlRTVzV2xWU2F6bG9ZVEJaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{AC193949-535B-4A89-9F7C-293D040801C4}"/>
-    <hyperlink ref="AL322" r:id="rId149" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFaVVZuaFZiRkpQVkRKV2MxWllhRlZXVmtwSFdsWlZlRlpXV2xWVmF6Vm9Za1ZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{91E9A798-28B7-4948-82E6-27F0D10D9096}"/>
-    <hyperlink ref="AL323" r:id="rId150" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFaVVZUSlZiRkpQVkRKV2MxWllaRlZOUmtwaFdsZHplR05YUmpaVmJFSlhVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{335B2C28-26D7-4B1C-A178-9F3D296B2F30}"/>
-    <hyperlink ref="AL325" r:id="rId151" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFaVWJGWlZiRkpQVkRKV2MxWllaRlZOUmtweFdsWlZlRlpXYkRaVGF6VnNZa1ZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{F4F69C17-3489-4845-B750-0270DCE1C958}"/>
-    <hyperlink ref="AL330" r:id="rId152" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYTAxRVZrWlZiRkpQVkRKV2MxWllaRlZOVmtwVFZGWlZNV05YUlhwaFJUVlRVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{0711F57B-B1F4-4905-A413-F6304C530753}"/>
-    <hyperlink ref="AL332" r:id="rId153" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYTAxRVZuaFZiRkpQVkRKV2MxWllaRlZOVmtwMVZGZHplRTVzVWxWU2JFSlhVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{DF9C1914-CF6E-4864-B5BB-43FFF5126F89}"/>
-    <hyperlink ref="AL334" r:id="rId154" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYTAxRWJFWlZiRkpQVkRKV2MxWllaRlZOVmtwNVdsVlZNVTVzYTNwalJUbFRVak5SZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{E6E8B2E3-8517-4B74-A113-10A62C544574}"/>
-    <hyperlink ref="AL337" r:id="rId155" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkZKVVJuaFZiRkpQVkRKV2MxWllhRlZXVmtweFZGVlZNVTVzU2xWVmJFSlhVak5SZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{B4B42B4E-04B1-4FB1-A253-6DE9A47CB643}"/>
-    <hyperlink ref="AL338" r:id="rId156" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkZKVVJUSlZiRkpQVkRKV2MxWllaRlZOVmtweFZGVlZNVlpXU2xWVWF6bG9Za1paZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{D44F7EF6-B201-4E62-9083-C17626447203}"/>
-    <hyperlink ref="AL342" r:id="rId157" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkZKVVZUSlZiRkpQVkRKV2MxWllhRlZXVmtweFZHdFZlRlpXYTNwaFJUVnNZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{986A6AB6-060B-4C3F-A942-B214ECF25664}"/>
-    <hyperlink ref="AL343" r:id="rId158" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkZKVWJFWlZiRkpQVkRKV2MxWllhRlZXVmtwVFdsWlZlRkpXUmxWUmF6bFhVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{EF80DAFC-0018-43A8-9EB1-0378FAC119A9}"/>
-    <hyperlink ref="AL344" r:id="rId159" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkZKVWJGWlZiRkpQVkRKV2MxWllhRlZXVmtweFZGWlZlRlpXYjNwYVJUbG9ZWHBGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{42F26756-4413-4DC8-8789-743629938E92}"/>
-    <hyperlink ref="AL346" r:id="rId160" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkZaVVJuaFZiRkpQVkRKV2MxWllhRlZXVmtwUFZGVlZlRTVzV2xWV2F6bG9Za1ZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{1D45023D-9254-4637-9F21-F0504498AB4A}"/>
-    <hyperlink ref="AL354" r:id="rId161" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkdGNlJuaFZiRkpQVkRKV2MxWllaRlZOUmtwVFZGUkJlRkpXVGxsaFJrSlRVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{3AB56B0D-D1F1-472F-AD42-55D666693344}"/>
-    <hyperlink ref="AL355" r:id="rId162" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkdGNlJUSlZiRkpQVkRKV2MxWllaRlZOVmtwSFZHdFZOVkpXY0RaU2F6bHNZWHBGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{6DE9EB2B-7B88-4907-B823-9EEAAF82AC29}"/>
-    <hyperlink ref="AL356" r:id="rId163" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkdGNlZrWlZiRkpQVkRKV2MxWllhRlZXVmtwUFdsVlZNVlpXVmxWU2JFSlRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{97DCDF91-0FBC-4AE7-B98E-97897A28CE44}"/>
-    <hyperlink ref="AL357" r:id="rId164" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkdGNlZsWlZiRkpQVkRKV2MxWllaRlZOUmtwMVdsVlZNVlpXV2xWVWF6Vm9Za1paZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{4A7BD6D1-0CF0-45DA-B924-5FEDE5BF7521}"/>
-    <hyperlink ref="AL358" r:id="rId165" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkdGNlZuaFZiRkpQVkRKV2MxWllhRlZXVmtwWFZGZHpNVkpXVWxWVmF6bG9ZVEZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{20C6FDDB-D146-48EA-8D96-9DF2BF5713DB}"/>
-    <hyperlink ref="AL364" r:id="rId166" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxKVVJUSlZiRkpQVkRKV2MxWllaRlZOVmtwWFZHdFZNV05XV2xsYVJrSlRVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{28F1130E-1B80-4278-9B29-EE12FDC8D8A3}"/>
-    <hyperlink ref="AL365" r:id="rId167" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxKVVZuaFZiRkpQVkRKV2MxWllaRlZOVmtwWFdsWlZlRTVzVWxWVmJFSlRVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{5688D473-D600-407B-95B5-DA94A7DEF4B9}"/>
-    <hyperlink ref="AL366" r:id="rId168" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxKVVZUSlZiRkpQVkRKV2MxWllaRlZOVmtwMVZGWlZlRlpXY0RaVmF6VnNZa2QzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{2877AA95-3FCD-453B-A87C-56E0220887EE}"/>
-    <hyperlink ref="AL367" r:id="rId169" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxKVWJFWlZiRkpQVkRKV2MxWllhRlZXVmtwaFZHeFZNV05XVmxsYVJUVm9ZVEZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{5FED4590-5708-470C-A832-B8F720A2AEF2}"/>
-    <hyperlink ref="AL369" r:id="rId170" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxaVVJsWlZiRkpQVkRKV2MxWllaRlZpYmtKMVZGUkJlRTVzV2xWUmF6bHNZa1paZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{601FEA6D-AC61-4968-B49D-0C962681E128}"/>
-    <hyperlink ref="AL370" r:id="rId171" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxaVVJUSlZiRkpQVkRKV2MxWllaRlZOUmtwNVdrUkJNVlpXWkZWUmF6VlhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{05EFC23E-890A-4E44-B266-368FA2E65C0B}"/>
-    <hyperlink ref="AL372" r:id="rId172" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxaVVZuaFZiRkpQVkRKV2MxWllaRlZpYmtKNVZGVlZNVlpYUmpaU2F6VnNZWHBGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{EA92E5EB-846F-4A1E-B002-AAB543A09D03}"/>
-    <hyperlink ref="AL373" r:id="rId173" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxaVVZUSlZiRkpQVkRKV2MxWllaRlZOUmtwRFZGZHplR05XYkRaVmF6bFhVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A4E30857-5D8A-404B-809E-811D0DE00E61}"/>
-    <hyperlink ref="AL374" r:id="rId174" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxaVWJFWlZiRkpQVkRKV2MxWllaRlZOUmtwRFdsVlZlRkpXWkZsYVJUbFRVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{EE7AC495-7FBE-4A28-A4F7-68715D1B25D3}"/>
-    <hyperlink ref="AL375" r:id="rId175" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVG1GNlJsWlZiRkpQVkRKV2MxWllaRlZOUmtwTFZGUkJNV05XVGxWVGF6VlRVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{E7CFD2F7-C9BF-43D1-BE94-71639B849034}"/>
-    <hyperlink ref="AL376" r:id="rId176" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVG1GNlJuaFZiRkpQVkRKV2MxWllaRlZOVmtwUFZGUkJOVlpXV2xWUmF6bFhVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{C836AA27-7E39-4B2B-BCEB-6E59A106EEDF}"/>
-    <hyperlink ref="AL377" r:id="rId177" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVG1GNlJUSlZiRkpQVkRKV2MxWllaRlZOUmtwUFZGVlZOVkpXVmxWVmJFSlhVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{0964BC11-0E5B-461B-BF2B-B0D2B078F5FF}"/>
-    <hyperlink ref="AL378" r:id="rId178" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVG1GNlZrWlZiRkpQVkRKV2MxWllaRlZOVmtwTFZHdFZNV05XWkZWV2F6bHNZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A441C873-3513-48C0-8917-2D2C973713FD}"/>
-    <hyperlink ref="AL380" r:id="rId179" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVG1GNlZuaFZiRkpQVkRKV2MxWllaRlZOVmtwTFdsZHpOVkpXVWxsaFJUVlRVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{CAEC4C01-DFD5-42FB-91DF-71B419027502}"/>
-    <hyperlink ref="AL381" r:id="rId180" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVG1GNlZUSlZiRkpQVkRKV2MxWllaRlZOVmtwTFdsVlZNVlpXVGxWVmF6bFhVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{21106479-95F1-4D99-AE2A-C8E77CC5D553}"/>
-    <hyperlink ref="AL383" r:id="rId181" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGsxRVJUSlZiRkpQVkRKV2MxWllaRlZOVmtwTFZGWlZlRTVzVGxWV2F6bG9ZWHBGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{B86F0C8F-76F5-4483-8DB5-7490674D429E}"/>
-    <hyperlink ref="AL384" r:id="rId182" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGsxRVZrWlZiRkpQVkRKV2MxWllhRlZXVmtwaFZGZHpNVTVzU2xWV2F6bFhVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{46D6A68A-17D3-4EFF-B764-FB770DDF6F94}"/>
-    <hyperlink ref="AL385" r:id="rId183" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGsxRVZsWlZiRkpQVkRKV2MxWllhRlZXVmtwWFZHdFZNVkpXY0RaV2F6VlhVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{872E86F2-8990-409D-B866-D198F5458283}"/>
-    <hyperlink ref="AL386" r:id="rId184" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGsxRVZuaFZiRkpQVkRKV2MxWllaRlZOVmtwVFdsWlZlRTV0UlhwaFJUVnNZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{056D38A3-E72C-46A1-901B-6EC72DF5376C}"/>
-    <hyperlink ref="AL387" r:id="rId185" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGsxRVZUSlZiRkpQVkRKV2MxWllaRlZOVmtwVFZGZHpNVTVzV2xWVWJFSlRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{33D12F19-7AAD-4ED2-B660-D0EEC1283158}"/>
-    <hyperlink ref="AL388" r:id="rId186" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGsxRWJFWlZiRkpQVkRKV2MxWllhRlZXVmtweFdsZHpOVlpXVGxWVmF6bFRVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{900BA918-5E69-485C-9B6C-203A532C6DEE}"/>
-    <hyperlink ref="AL391" r:id="rId187" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVDFKVVZrWlZiRkpQVkRKV2MxWllhRlZXYkVwRFdsWlZlRTVzVmxWVWF6VlhVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{FD7E43B6-5E49-4537-B5C0-D9A5B8C00C45}"/>
-    <hyperlink ref="AL395" r:id="rId188" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVDFaVVJrWlZiRkpQVkRKV2MxWllaRlZOVmtwUFZHdFZOVlpXU2xsaVJUbG9Za1ZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{FE9C368C-A3B4-48D2-8232-CEE6229FEBC4}"/>
-    <hyperlink ref="AL396" r:id="rId189" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVDFaVVJsWlZiRkpQVkRKV2MxWllaRlZOVmtwTFZGWlZlR05XVWxsaVJUbHNZbGRSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A14893FB-1B90-4282-8186-CAAFC594DB95}"/>
-    <hyperlink ref="AL425" r:id="rId190" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkZKVVJrWlZiRkpQVkRKV2MxWllaRlZOUmtwaFdsWlZlR05XVWxsaVJUbFhVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{07467D07-0152-4F98-9D06-AA0FB5DE4EA2}"/>
-    <hyperlink ref="AL436" r:id="rId191" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxKVVZrWlZiRkpQVkRKV2MxWllaRlZOVmtwSFZGUkJNV05XYTNwaVJUbG9Za1ZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{0456CBCA-FB41-4768-9CFC-FD801A90385D}"/>
-    <hyperlink ref="AL438" r:id="rId192" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzAxVDFKVVZUSlZiRkpQVkRKV2MxWllaRlZOVmtwTFdsWlZNVTVzVWxWV2F6Vm9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{9325C63C-E328-4C00-A5D6-830A88CE95FA}"/>
-    <hyperlink ref="AL442" r:id="rId193" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlpZMFZLVDFKVVZUSlZiRkpQVkRKV2MxWllaRlZOVmtwMVZHdFZlRTV0UmpaVmF6VnNZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{9D111EAD-5447-4040-9B5B-D3681493BA82}"/>
-    <hyperlink ref="AL445" r:id="rId194" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlpZMFZLVDFaVVJrWlZiRkpQVkRKV2MxWllaRlZOVmtwWFZGWlZNVTVzVWxWVmF6VlRVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{6C772F02-B6C9-4C91-BF80-0711FBAB0FDA}"/>
-    <hyperlink ref="AL449" r:id="rId195" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlpZMFZLVDFaVVZrWlZiRkpQVkRKV2MxWllaRlZOVmtwTFdsWlZlR05XUmxWVWF6VlRVakEwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{0CCBE737-864E-4E83-AFDF-C022C935A5F9}"/>
-    <hyperlink ref="AL452" r:id="rId196" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlpZMFZLVDFaVVZUSlZiRkpQVkRKV2MxWllhRlZXVmtwSFZHdFZlRTVzU2xWV2F6VlhVakEwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{F8D3B610-E14A-4630-B13E-DC4B0D9C97D6}"/>
-    <hyperlink ref="AL499" r:id="rId197" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528380&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSnlWV3MxYkdGNlJrWlZiRkpQVkRKV2MxWllaRlZOUmtwNVZGVlZlR05XYjNwalJUbFhVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{6FD65F5B-9608-43D1-8BA9-6043436F9358}"/>
+    <hyperlink ref="AL14" r:id="rId1" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528591&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzAxVG1GNlZrWlZiRkpQVkRKV2MxWllaRlZOVmtwUFdsVlZOVlpXV2xsaVJrSlRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{83556729-D731-48CF-BD8D-B04618F7138D}"/>
+    <hyperlink ref="AL22" r:id="rId2" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528591&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkZKVVZsWlZiRkpQVkRKV2MxWllaRlZOUmtwVFZGVlZNV05XVGxWUmF6VlRVak5SZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{77482D17-1FCE-4BD4-A22E-D50C8C56C803}"/>
+    <hyperlink ref="AL25" r:id="rId3" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528591&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkZaVVJsWlZiRkpQVkRKV2MxWllaRlZOVmtwSFdsWlZOVlpXV2xWUmF6VlRVak5SZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{EE82EF45-084F-449A-B29E-B14E1B5FE615}"/>
+    <hyperlink ref="AL26" r:id="rId4" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528591&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkZaVVJuaFZiRkpQVkRKV2MxWllaRlZOVmtwTFZGUkJNVTVzVmxsaFJUVlRVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{05210B84-F679-49B1-A3E7-182BA9B9D2B2}"/>
+    <hyperlink ref="AL29" r:id="rId5" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528591&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkZaVVZuaFZiRkpQVkRKV2MxWllhRlZXYkVwRFZGZHplRkpXVGxWVGF6Vm9ZbGRSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{AF710FA1-A605-4618-A1B0-DE218AB4AFFC}"/>
+    <hyperlink ref="AL30" r:id="rId6" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528591&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkZaVVZUSlZiRkpQVkRKV2MxWllhRlZXYkVwRFZGWlZNVlpXVGxsYVJrSlhVak5SZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{CC27D715-755E-482C-AF91-D4E80DA1A2F6}"/>
+    <hyperlink ref="AL32" r:id="rId7" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528591&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkdGNlJrWlZiRkpQVkRKV2MxWllhRlZXYkVwSFdsWlZlRTVzV2xsYVJUbFhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{3D585F5C-0399-457B-8C5D-73FB21B7B2DC}"/>
+    <hyperlink ref="AL33" r:id="rId8" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528591&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkdGNlJsWlZiRkpQVkRKV2MxWllaRlZOUmtwSFZGWlZNVkpXY0RaU2F6VnNZa2QzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{7BB46791-B143-4DED-9CB7-6CC5C7FB1FBB}"/>
+    <hyperlink ref="AL39" r:id="rId9" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528591&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkdGNmJFWlZiRkpQVkRKV2MxWllhRlZXVmtwaFZHdFZNV05XVmxWVmF6bG9ZbGRSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{0698E7B5-1418-4982-8B7D-35720A92DD75}"/>
+    <hyperlink ref="AL40" r:id="rId10" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528591&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkdGNmJGWlZiRkpQVkRKV2MxWllhRlZXVmtwVFZHdFZlRTVzWkZsalJUVm9ZVEZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{004D7BD8-A2CE-482D-B192-0AE8AF751532}"/>
+    <hyperlink ref="AL41" r:id="rId11" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528591&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGxKVVJrWlZiRkpQVkRKV2MxWllhRlZXVmtwWFdsWlZOVlpXWkZsalJUVlRVakEwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{D8EAEC77-42E6-467C-8B61-FE84F043E88C}"/>
+    <hyperlink ref="AL42" r:id="rId12" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528591&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGxKVVJuaFZiRkpQVkRKV2MxWllaRlZOVmtwUFZGWlZNV05XVmxWUmF6Vm9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{D2732984-80BF-477C-A12C-3EA7451DA10C}"/>
+    <hyperlink ref="AL44" r:id="rId13" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528591&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGxKVVZrWlZiRkpQVkRKV2MxWllaRlZOVmtwUFZGUkJOVlpXVmxsalJUbHNZa2QzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{0AE59120-CDA7-41C2-8C7C-7CB72ABD871A}"/>
+    <hyperlink ref="AL45" r:id="rId14" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528591&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGxKVVZsWlZiRkpQVkRKV2MxWllaRlZOVmtwUFZHeFZOVkpXU2xWV2F6VlhVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{44985175-2696-41D3-9554-87BBB9F29DA5}"/>
+    <hyperlink ref="AL46" r:id="rId15" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528591&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGxKVVZuaFZiRkpQVkRKV2MxWllaRlZOVmtwUFZGWlZlRTVzVWxsalJUbFRVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{306C3375-E12C-4488-A048-6EE21D4CA759}"/>
+    <hyperlink ref="AL47" r:id="rId16" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528591&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGxKVVZUSlZiRkpQVkRKV2MxWllaRlZOUmtwTFdsZHpNVTVzVGxsYVJUVlhVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A0A9B0D9-9F9A-4B25-B270-71AC1ABE9370}"/>
+    <hyperlink ref="AL50" r:id="rId17" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGxaVVJrWlZiRkpQVkRKV2MxWllaRlZOUmtwTFZGVlZOVkpXYkRaVGJFSlRVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{8F0A3B24-9F72-4C0F-A7BD-45D4FB633DF9}"/>
+    <hyperlink ref="AL52" r:id="rId18" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGxaVVJuaFZiRkpQVkRKV2MxWllhRlZXVmtwWFZGZHpNVTV0UmpaUmF6bHNZa1ZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{94307207-34A7-4C63-A2C9-383B471393A7}"/>
+    <hyperlink ref="AL53" r:id="rId19" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGxaVVJUSlZiRkpQVkRKV2MxWllhRlZXYkVwRFdsZHplRkpXUmxsaVJUVm9Za1ZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{B7C5EF1D-DEA6-41F5-A677-4AAE794912DD}"/>
+    <hyperlink ref="AL59" r:id="rId20" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVG1GNlJrWlZiRkpQVkRKV2MxWllhRlZXYkVwSFdsWlZNVkpXY0RaUmJFSlhVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{760BE2F5-007A-40E6-9EC7-6F7ABDCE8594}"/>
+    <hyperlink ref="AL60" r:id="rId21" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVG1GNlJsWlZiRkpQVkRKV2MxWllaRlZOUmtwWFZGWlZNV05XVmxWUmF6bFRVakEwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{E8919FD4-A348-4822-BF16-4D1E4F925C5B}"/>
+    <hyperlink ref="AL62" r:id="rId22" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVG1GNlJUSlZiRkpQVkRKV2MxWllaRlZOVmtwVFZGUkJNVkpXVWxWU2F6bG9ZVEJaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{8EF47378-AB63-455E-A00C-2C2536105F5A}"/>
+    <hyperlink ref="AL63" r:id="rId23" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVG1GNlZrWlZiRkpQVkRKV2MxWllaRlZOVmtwVFdrUkJlR05XV2xWVmJFSlhVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{22F238F2-E2DD-497B-AFE8-3234DC4D3318}"/>
+    <hyperlink ref="AL65" r:id="rId24" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVG1GNlZuaFZiRkpQVkRKV2MxWllaRlZOVmtwTFZGVlZlRlpXWkZsaVJUbFRVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{F8FB8ADA-2873-43BE-90E1-1DF6B742F0B7}"/>
+    <hyperlink ref="AL67" r:id="rId25" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVG1GNmJFWlZiRkpQVkRKV2MxWllhRlZXYkVwRFZHdFZOVlpXUmxWVWF6VlRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{3809C15A-5B5B-4245-8BD3-6B8A42C73D5C}"/>
+    <hyperlink ref="AL68" r:id="rId26" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVG1GNmJGWlZiRkpQVkRKV2MxWllaRlZOVmtweFdsZHplRTVzVmxWVmF6bFhVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A26AD090-3B1A-48A5-9A9F-C57916E827B7}"/>
+    <hyperlink ref="AL69" r:id="rId27" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGsxRVJrWlZiRkpQVkRKV2MxWllhRlZXVmtwaFdsZHpNV05YUlhwalJUbFhVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{8EC92629-4C9A-4F46-BC86-9C2B6B1235C0}"/>
+    <hyperlink ref="AL70" r:id="rId28" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGsxRVJsWlZiRkpQVkRKV2MxWllaRlZOVmtwNVdsZHpNVkpXV2xsaFJUbFRVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{64B0BBAC-B2C2-42D3-BDDB-18ABAA74627B}"/>
+    <hyperlink ref="AL73" r:id="rId29" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGsxRVZrWlZiRkpQVkRKV2MxWllhRlZXYkVwSFZHdFZNVlpXVWxWVmF6bG9ZWHBGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{CD5FFDFB-24B4-4B0D-BA30-E6D736149483}"/>
+    <hyperlink ref="AL77" r:id="rId30" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVGsxRWJFWlZiRkpQVkRKV2MxWllaRlZOVmtwTFZGZHpOVlpXU2xsalJUbFRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{2B9C969A-291A-4874-B551-5370DBFBA427}"/>
+    <hyperlink ref="AL82" r:id="rId31" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVDFKVVJUSlZiRkpQVkRKV2MxWllhRlZXVmtwSFdsZHpOVlpXVmxsalJUVnNZWHBGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{6DCB0778-CEFE-4CF8-B449-1EDB73BC97DC}"/>
+    <hyperlink ref="AL83" r:id="rId32" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVDFKVVZrWlZiRkpQVkRKV2MxWllaRlZOUmtwaFZGZHpOVkpXVmxsYVJUVlhVak5SZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{6A1A08A9-0E6B-4ECF-989A-43B361EE85A3}"/>
+    <hyperlink ref="AL87" r:id="rId33" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVDFaVVJsWlZiRkpQVkRKV2MxWllhRlZXVmtweFdsWlZlR05XVGxsalJUbFRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{6F353D0D-F66B-4F95-9DD2-424F584CA8A7}"/>
+    <hyperlink ref="AL88" r:id="rId34" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVDFaVVJuaFZiRkpQVkRKV2MxWllaRlZOVmtwMVZGVlZNV05XVWxsalJUVlRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{E052C995-80E1-48B7-9225-3F5077ED004B}"/>
+    <hyperlink ref="AL89" r:id="rId35" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVDFaVVJUSlZiRkpQVkRKV2MxWllaRlZOVmtwUFdsVlZlRTVzVWxWVGJFSlRVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{2B880630-AF3E-4BC0-9A48-D2DE28B1D2EC}"/>
+    <hyperlink ref="AL90" r:id="rId36" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLVDFaVVZrWlZiRkpQVkRKV2MxWllaRlZOUmtwaFZGWlZNVlpXWkZWVGF6bG9ZVEZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{F7F30B9A-9717-47E7-9EF9-DCB1B12C6F31}"/>
+    <hyperlink ref="AL98" r:id="rId37" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYTAxRVZrWlZiRkpQVkRKV2MxWllaRlZOUmtwSFZHeFZlR05XY0RaV2F6VlRVak5SZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{CAAE9088-9D48-4FF9-8FEF-4853A6D4170A}"/>
+    <hyperlink ref="AL103" r:id="rId38" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYTAxRWJGWlZiRkpQVkRKV2MxWllaRlZOUmtwSFZHeFZlRkpXWkZWVGF6bHNZbGhSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{38D74FA8-F2CF-4F5E-B76E-93F5383FDABE}"/>
+    <hyperlink ref="AL104" r:id="rId39" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZKVVJrWlZiRkpQVkRKV2MxWllhRlZXVmtwTFZGWlZlRkpXVWxWVmF6VnNZVEJaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{D893522E-490C-431E-B1FD-53B2164A2D57}"/>
+    <hyperlink ref="AL107" r:id="rId40" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZKVVJUSlZiRkpQVkRKV2MxWllhRlZXVmtwWFZGZHpNVTVzWkZWV2F6bFRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{3274FCFC-60D6-4F0A-B069-8E66F446943E}"/>
+    <hyperlink ref="AL108" r:id="rId41" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZKVVZrWlZiRkpQVkRKV2MxWllaRlZOUmtwRFdsZHpNVTVzUmxsYVJUbHNZVEZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{FC905051-53BD-4FA9-9831-724028A5B917}"/>
+    <hyperlink ref="AL109" r:id="rId42" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZKVVZsWlZiRkpQVkRKV2MxWllaRlZOUmtwSFdrUkJlRlpXU2xWVmF6bFhVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A7246DBC-6721-4816-9F5F-EE5011AD9B7F}"/>
+    <hyperlink ref="AL110" r:id="rId43" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZKVVZuaFZiRkpQVkRKV2MxWllhRlZXYkVwTFdrUkJlRlpXUmxsaFJUbFhVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{C208589A-140A-4246-ACDE-918D41A451FA}"/>
+    <hyperlink ref="AL111" r:id="rId44" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZKVVZUSlZiRkpQVkRKV2MxWllaRlZpYmtKeFZGZHpNVlpXWkZsalJUVm9Za2QzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{3D9996CF-E2BE-4989-B114-D9A1FFC8017E}"/>
+    <hyperlink ref="AL112" r:id="rId45" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZKVWJFWlZiRkpQVkRKV2MxWllaRlZpYmtKMVZGVlZNVTVzYkRaU2F6VlRVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{3E4FF25E-CD1C-4857-92CD-605F79B2C305}"/>
+    <hyperlink ref="AL115" r:id="rId46" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZaVVJsWlZiRkpQVkRKV2MxWllaRlZOVmtwVFdsVlZlRkpXUmxsaFJUbFhVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{AF7A4F71-2D6A-4D30-A030-015BAC8422BA}"/>
+    <hyperlink ref="AL119" r:id="rId47" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZaVVZsWlZiRkpQVkRKV2MxWllhRlZXVmtwUFZGUkJOVkpXYjNwalJUbG9ZbGhSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{177F6FA9-2414-4ED1-B2ED-F839A1ED1445}"/>
+    <hyperlink ref="AL120" r:id="rId48" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZaVVZuaFZiRkpQVkRKV2MxWllaRlZOVmtwVFdsVlZNVlpXVmxsaVJUbFRVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A9F14308-E804-4A81-AFE2-9EC2521C5ACE}"/>
+    <hyperlink ref="AL121" r:id="rId49" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZaVVZUSlZiRkpQVkRKV2MxWllaRlZOVmtwNVZGVlZlRlpXVWxWVmF6Vm9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{F02626DD-5350-45DA-8732-2C00BC8DD95C}"/>
+    <hyperlink ref="AL122" r:id="rId50" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZaVWJFWlZiRkpQVkRKV2MxWllhRlZXVmtwNVZGUkJOVlpXUmxWVGF6bHNZa2QzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{224791D7-D4FB-452C-8A6E-B330A32D8467}"/>
+    <hyperlink ref="AL123" r:id="rId51" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkZaVWJGWlZiRkpQVkRKV2MxWllaRlZOVmtwUFZGZHpNVkpXYjNwYVJUbFRVakEwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{5C9CB204-88DB-4E7B-B585-5729A824E073}"/>
+    <hyperlink ref="AL125" r:id="rId52" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkdGNlJsWlZiRkpQVkRKV2MxWllaRlZOUmtwSFZGUkJlR05XVWxsaFJUVm9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{08A0F1AE-0882-4AEE-9F72-60E197C67EF1}"/>
+    <hyperlink ref="AL126" r:id="rId53" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkdGNlJuaFZiRkpQVkRKV2MxWllaRlZOVmtwUFZGUkJOVlpXVWxsaFJUbHNZbGRSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{5859C7C1-5FDF-477F-85E1-2AF87356B053}"/>
+    <hyperlink ref="AL127" r:id="rId54" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkdGNlJUSlZiRkpQVkRKV2MxWllaRlZOUmtwTFZHeFZOVkpXUmxsYVJUVlRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A361A311-9085-427C-BFB6-A19A317A4FD0}"/>
+    <hyperlink ref="AL128" r:id="rId55" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkdGNlZrWlZiRkpQVkRKV2MxWllaRlZpYmtKNVdsZHplRTVzV2xWVmJFSlRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{226B1B67-E524-4D85-AB3B-72FDF2AF8035}"/>
+    <hyperlink ref="AL129" r:id="rId56" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkdGNlZsWlZiRkpQVkRKV2MxWllaRlZOUmtwRFdsZHpNVkpXYTNwalJUbFhVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{9B2D1F62-D9C5-4DF3-BA66-76F2E108E24E}"/>
+    <hyperlink ref="AL131" r:id="rId57" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkdGNlZUSlZiRkpQVkRKV2MxWllhRlZXVmtwMVZHeFZlR05XVmxWVWJFSlRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{E234EA54-5CDE-430A-98C1-DD76DDF00F51}"/>
+    <hyperlink ref="AL132" r:id="rId58" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkdGNmJFWlZiRkpQVkRKV2MxWllhRlZXVmtwMVZGWlZlRTVzV2xWVWJFSlhVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{B95D2A24-89FF-489A-8E2E-6DAB71325ED4}"/>
+    <hyperlink ref="AL133" r:id="rId59" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLYkdGNmJGWlZiRkpQVkRKV2MxWllhRlZXVmtwMVdrUkJOVkpXVWxsYVJUVm9ZbGhSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{F1018EC9-1CCD-4B36-B5F9-F1A3E325A591}"/>
+    <hyperlink ref="AL134" r:id="rId60" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxKVVJrWlZiRkpQVkRKV2MxWllhRlZXVmtwaFdsZHplR05XYkRaU2F6VlRVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{89EFAE0E-0D35-4C05-A2F9-00F0A5635958}"/>
+    <hyperlink ref="AL136" r:id="rId61" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxKVVJuaFZiRkpQVkRKV2MxWllaRlZOUmtwRFZHdFZlR05YUmpaUmF6bFhVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{DF000B7E-FE91-4A52-B148-55803145AF72}"/>
+    <hyperlink ref="AL138" r:id="rId62" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxKVVZsWlZiRkpQVkRKV2MxWllaRlZOVmtwRFZGWlZNVkpXU2xWV2F6bFRVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{7B635850-7CBF-4C19-A0AE-B4E346CF6191}"/>
+    <hyperlink ref="AL139" r:id="rId63" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxKVVZuaFZiRkpQVkRKV2MxWllaRlZOUmtweFdsVlZlRlpXVmxWVWF6bHNZbGhSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{FB6D7F6B-5F6A-4DDE-8883-F8821C343997}"/>
+    <hyperlink ref="AL140" r:id="rId64" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxKVVZUSlZiRkpQVkRKV2MxWllaRlZOUmtweFdsZHpOVlpXU2xsalJUbFRVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{8F399858-923E-4306-BA61-7BD8E2E04AD6}"/>
+    <hyperlink ref="AL142" r:id="rId65" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxKVWJGWlZiRkpQVkRKV2MxWllaRlZOVmtwWFdrUkJOVkpXV2xWVWF6bFhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{B4629DD4-ED46-4203-A5E7-954622CA43D1}"/>
+    <hyperlink ref="AL144" r:id="rId66" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxaVVJsWlZiRkpQVkRKV2MxWllaRlZOVmtwTFdsVlZOVlpYUmpaVGF6bFhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{1608605A-487E-43B5-99D9-529E324951E3}"/>
+    <hyperlink ref="AL146" r:id="rId67" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxaVVJUSlZiRkpQVkRKV2MxWllhRlZXVmtweFdsZHpNV05XVmxsaVJrSlRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{3CFE27B7-8833-4651-8A3B-BF4E37318ED8}"/>
+    <hyperlink ref="AL149" r:id="rId68" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxaVVZuaFZiRkpQVkRKV2MxWllaRlZOUmtwUFZGWlZNVkpXYkRaU2F6VnNZa2QzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{99F5A94F-1B82-45F0-9691-943AA2626F55}"/>
+    <hyperlink ref="AL151" r:id="rId69" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGxaVWJFWlZiRkpQVkRKV2MxWllaRlZOUmtwaFdrUkJOVlpXVmxsaFJUbG9Za1paZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{CEB51617-385D-41EA-9EF5-104434B00329}"/>
+    <hyperlink ref="AL153" r:id="rId70" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVG1GNlJrWlZiRkpQVkRKV2MxWllaRlZOUmtwTFZGWlZlR05XVWxsalJUbG9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{3B0DB09F-AEAF-418C-A9E4-9F7F18B09431}"/>
+    <hyperlink ref="AL155" r:id="rId71" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVG1GNlJuaFZiRkpQVkRKV2MxWllhRlZXVmtwTFZHeFZlRkpXUmxsaVJUbG9ZWHBGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{36EF42BA-1110-4771-8538-130EB7191B88}"/>
+    <hyperlink ref="AL160" r:id="rId72" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVG1GNmJFWlZiRkpQVkRKV2MxWllaRlZOVmtwSFdrUkJlR05XVmxWVGF6VlhVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{B1E207D4-56F0-4DED-9D65-F4A9C002F7CC}"/>
+    <hyperlink ref="AL161" r:id="rId73" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVG1GNmJGWlZiRkpQVkRKV2MxWllhRlZXVmtwVFZHeFZNVkpXU2xsaVJUVlRVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{89374AD4-3495-4F3A-8C34-81482631BE6E}"/>
+    <hyperlink ref="AL163" r:id="rId74" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGsxRVJsWlZiRkpQVkRKV2MxWllhRlZXVmtwTFdsZHpNVTVzVGxWVmF6VlhVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{065BA9B9-2DFC-4966-99AD-4B65E07F31EA}"/>
+    <hyperlink ref="AL166" r:id="rId75" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGsxRVZrWlZiRkpQVkRKV2MxWllhRlZXVmtwVFdrUkJNVlpXYjNwalJUbFhVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{EEFDACF5-35D8-45F3-B00B-D3512A255269}"/>
+    <hyperlink ref="AL168" r:id="rId76" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGsxRVZuaFZiRkpQVkRKV2MxWllaRlZOVmtwUFdsVlZlRkpXVmxsalJUbFhVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{7A8C25AD-235E-46E1-9FEA-379E5AE31B0B}"/>
+    <hyperlink ref="AL171" r:id="rId77" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVGsxRWJGWlZiRkpQVkRKV2MxWllaRlZOVmtwTFdsZHpNV05XY0RaUmF6Vm9ZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{7B496C1A-5090-4984-83B2-3B84E8234B05}"/>
+    <hyperlink ref="AL172" r:id="rId78" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVDFKVVJrWlZiRkpQVkRKV2MxWllhRlZXVmtwVFZGUkJlRlpXV2xWVGF6bFhVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{03D95577-1DD1-4A2C-979E-A1CA83E5BFC7}"/>
+    <hyperlink ref="AL176" r:id="rId79" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVDFKVVZrWlZiRkpQVkRKV2MxWllhRlZXVmtwMVZHeFZNVTVzYTNwaFJUbFhVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{EA7AEAD4-69AD-4184-AE6A-523A0010C431}"/>
+    <hyperlink ref="AL177" r:id="rId80" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVDFKVVZsWlZiRkpQVkRKV2MxWllaRlZOVmtwWFZGVlZlRlpXV2xsYVJUbFhVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{315C273E-87AC-4479-91B0-A4E01A060FF2}"/>
+    <hyperlink ref="AL178" r:id="rId81" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVDFKVVZuaFZiRkpQVkRKV2MxWllaRlZOUmtwMVZGVlZOVkpXYTNwaVJUVlhVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{93EF5CA7-A453-4314-9DE0-0AA3C572A3DF}"/>
+    <hyperlink ref="AL179" r:id="rId82" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVDFKVVZUSlZiRkpQVkRKV2MxWllaRlZOUmtwNVdsZHpOVlpXYkRaVmF6bHNZbGRSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A22FA17F-4A10-403B-AE9B-2423C816E6A1}"/>
+    <hyperlink ref="AL182" r:id="rId83" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVDFaVVJrWlZiRkpQVkRKV2MxWllaRlZpYmtKMVZGVlZlRkpXYkRaVmF6bFhVakEwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{6C0045C7-1C42-4CB7-95DD-8CCA0BF37359}"/>
+    <hyperlink ref="AL183" r:id="rId84" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVDFaVVJsWlZiRkpQVkRKV2MxWllhRlZXVmtwMVdsZHpOVkpXUmxWVmF6VlhVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{EE7C8822-4B47-4729-90E2-0EF73804A589}"/>
+    <hyperlink ref="AL186" r:id="rId85" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZLVDFaVVZrWlZiRkpQVkRKV2MxWllaRlZOVmtwaFdsVlZlRTVzVGxsaFJUVlRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{F7774577-3615-4FF6-B42A-10AC58756B58}"/>
+    <hyperlink ref="AL191" r:id="rId86" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYTAxRVJrWlZiRkpQVkRKV2MxWllaRlZOUmtwaFZGVlZOVkpXYTNwYVJUbG9ZbGhSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{3FB78DB4-DBB8-45F4-B8FB-F3FDCD360908}"/>
+    <hyperlink ref="AL192" r:id="rId87" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYTAxRVJsWlZiRkpQVkRKV2MxWllhRlZXYkVwSFdsZHplRkpYUmpaUmJFSlRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{85869DD6-ABEE-490C-9212-10E6AC8F92CF}"/>
+    <hyperlink ref="AL193" r:id="rId88" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYTAxRVJuaFZiRkpQVkRKV2MxWllaRlZOVmtwRFdsZHpNV05YUlhwYVJUbG9Za2QzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{EA77F3B4-1536-4FE2-9436-BF597D938265}"/>
+    <hyperlink ref="AL196" r:id="rId89" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYTAxRVZsWlZiRkpQVkRKV2MxWllaRlZOUmtwNVZGZHpOVkpXVmxsaFJUVnNZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{3620B269-BA21-4219-B743-53AD153FB6E3}"/>
+    <hyperlink ref="AL197" r:id="rId90" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYTAxRVZuaFZiRkpQVkRKV2MxWllaRlZOUmtwRFZGVlZNVlpXU2xWV2F6bG9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{59112182-F470-4383-A43D-F5E84D792D2B}"/>
+    <hyperlink ref="AL199" r:id="rId91" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYTAxRWJFWlZiRkpQVkRKV2MxWllaRlZOVmtwSFZGUkJOVlpXU2xsalJUbFhVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{240124A5-3DCC-42FC-8F56-5B7CFBFE1173}"/>
+    <hyperlink ref="AL201" r:id="rId92" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYkZKVVJrWlZiRkpQVkRKV2MxWllhRlZXVmtwVFZGZHplRlpXVGxWUmJFSlhVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{DDA71934-182E-407D-BCDB-E8E21D1D4A35}"/>
+    <hyperlink ref="AL203" r:id="rId93" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYkZKVVJuaFZiRkpQVkRKV2MxWllaRlZOUmtwNVdsVlZNVlpXVWxWV2F6VlhVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{005DEBBF-755C-4E19-A2E9-0D88B455AD07}"/>
+    <hyperlink ref="AL206" r:id="rId94" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYkZKVVZuaFZiRkpQVkRKV2MxWllhRlZXYkVwRFdsWlZlRlpXU2xsalJUbFhVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{04530E9E-B5B7-4BD0-B59E-5E13BE815446}"/>
+    <hyperlink ref="AL211" r:id="rId95" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYkZaVVJuaFZiRkpQVkRKV2MxWllaRlZOUmtwWFZGWlZlRlpXWkZsaFJUbG9ZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{B80A0FD7-828A-4962-AA1D-1A0644CE002B}"/>
+    <hyperlink ref="AL212" r:id="rId96" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYkZaVVZrWlZiRkpQVkRKV2MxWllaRlZOUmtwRFdsVlZlR05YUmpaVWJFSlhVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{D225241A-2072-42DF-A7BA-7733C81352E7}"/>
+    <hyperlink ref="AL221" r:id="rId97" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhYkdGNlZsWlZiRkpQVkRKV2MxWllaRlZOUmtwSFZGVlZNV05XWkZsYVJUbFhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{C7A3250B-90E6-48D5-8573-5A5A122B50BD}"/>
+    <hyperlink ref="AL226" r:id="rId98" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhVGxKVVZrWlZiRkpQVkRKV2MxWllaRlZOUmtwMVZGVlZOVlpXUmxWU2F6VnNZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{87C096E7-113B-43CB-A648-FC136FF0A143}"/>
+    <hyperlink ref="AL227" r:id="rId99" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhVGxKVVZsWlZiRkpQVkRKV2MxWllaRlZOVmtwWFdsWlZNVkpXVmxsaVJUbHNZVEJaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{FF45D65C-3960-48C9-8F8C-1753B29F0B21}"/>
+    <hyperlink ref="AL228" r:id="rId100" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFZhVGxKVVZuaFZiRkpQVkRKV2MxWllaRlZOVmtwVFdrUkJNVkpYUmpaU2F6bHNZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{C2B0D162-7CA0-43C4-8D4C-92C40FDA25C1}"/>
+    <hyperlink ref="AL232" r:id="rId101" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYTAxRVJuaFZiRkpQVkRKV2MxWllaRlZOUmtwWFZGZHplRTVzWkZWUmF6bFhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A2804D7E-9E1C-473E-832E-046A85C367B7}"/>
+    <hyperlink ref="AL233" r:id="rId102" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYTAxRVJUSlZiRkpQVkRKV2MxWllaRlZOUmtwaFZGUkJlRTVzVWxsalJUVlhVak5SZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{041A187F-ABCB-4031-A372-96F994809385}"/>
+    <hyperlink ref="AL234" r:id="rId103" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYTAxRVZrWlZiRkpQVkRKV2MxWllaRlZOUmtwMVZHdFZlRkpXWkZWVGJFSlhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{F6CA3CCC-6545-42F7-A814-A49A20575733}"/>
+    <hyperlink ref="AL235" r:id="rId104" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYTAxRVZsWlZiRkpQVkRKV2MxWllaRlZOUmtwaFdrUkJlRkpXVmxsYVJUVnNZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{3E65A60E-4D68-49EE-AE17-EF2425D10DF5}"/>
+    <hyperlink ref="AL236" r:id="rId105" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYTAxRVZUSlZiRkpQVkRKV2MxWllaRlZOVmtwMVZGVlZNVlpXVWxWVWF6bFhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{8594628B-520C-4077-BFB0-838725C12F53}"/>
+    <hyperlink ref="AL237" r:id="rId106" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYTAxRWJFWlZiRkpQVkRKV2MxWllhRlZXVmtwVFdsVlZNVTVzU2xsaFJUVlRVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{96EC8DBB-B420-4C31-A7B8-1007281B0CA6}"/>
+    <hyperlink ref="AL238" r:id="rId107" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYTAxRWJGWlZiRkpQVkRKV2MxWllhRlZXVmtweFdsVlZNVkpXVWxWUmF6bHNZbGhSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A7547B45-9676-45BD-A610-BC5059FF9F77}"/>
+    <hyperlink ref="AL239" r:id="rId108" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYkZKVVJrWlZiRkpQVkRKV2MxWllaRlZOUmtwUFZGZHplRlpXU2xWVGF6bG9ZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A5433B20-9FDF-4868-8345-071E2EB181F9}"/>
+    <hyperlink ref="AL243" r:id="rId109" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYkZKVVZrWlZiRkpQVkRKV2MxWllhRlZXVmtwMVdsWlZNV05XVWxWV2F6Vm9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{F3AD036E-2CA2-49E1-971F-A60CBA0FF1FC}"/>
+    <hyperlink ref="AL247" r:id="rId110" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYkZaVVJUSlZiRkpQVkRKV2MxWllhRlZXVmtwVFZGZHpOVkpXVmxWVGF6Vm9Za1paZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{5B0D33AC-7ED2-4759-9371-55ED3F19AAD9}"/>
+    <hyperlink ref="AL248" r:id="rId111" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYkZaVVZuaFZiRkpQVkRKV2MxWllhRlZXVmtwMVdsWlZlRTVzY0RaVWF6bFRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{33178571-18AE-43B0-9DF4-2E6D900A77BE}"/>
+    <hyperlink ref="AL249" r:id="rId112" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYkdGNlZsWlZiRkpQVkRKV2MxWllaRlZOVmtwSFZGWlZlR05XVGxWVGF6bHNZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{38509673-BED8-4E12-BE1D-4596B44D0B6A}"/>
+    <hyperlink ref="AL250" r:id="rId113" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYkdGNmJFWlZiRkpQVkRKV2MxWllhRlZXVmtwTFZGZHpOVlpXV2xsaFJUbFRVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{003D32F0-D139-420F-80E2-98A5B65EE145}"/>
+    <hyperlink ref="AL251" r:id="rId114" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxYkdGNmJGWlZiRkpQVkRKV2MxWllaRlZOVmtwUFZGWlZNVlpXUmxWVmF6bFhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{D02CFA32-D8A0-432C-8664-79DEE762818F}"/>
+    <hyperlink ref="AL252" r:id="rId115" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxVGxKVVJsWlZiRkpQVkRKV2MxWllaRlZOUmtweFdsVlZNVlpXVmxWVWF6bG9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{556149E0-7DE3-4BA9-9F33-6414C2420C77}"/>
+    <hyperlink ref="AL254" r:id="rId116" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxVGxKVVZrWlZiRkpQVkRKV2MxWllhRlZXVmtwMVdsVlZOVkpYUmpaVmF6bFhVak5SZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{3823EEC8-3463-4E3E-818A-6950866500C4}"/>
+    <hyperlink ref="AL255" r:id="rId117" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxVGxKVVZsWlZiRkpQVkRKV2MxWllhRlZXVmtwNVZGZHpOVlpYUlhwaFJUbG9ZWHBGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{8F04D773-3E2E-4886-9476-3320FC079B86}"/>
+    <hyperlink ref="AL256" r:id="rId118" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxVGxKVVZuaFZiRkpQVkRKV2MxWllhRlZXVmtwMVZGZHpNVkpXYjNwYVJUbFRVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{F41EA6FE-3EF2-4EFE-A051-8A448BE78321}"/>
+    <hyperlink ref="AL257" r:id="rId119" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFUxVGxKVVZUSlZiRkpQVkRKV2MxWllhRlZXVmtwNVdsWlZlRlpXY0RaU2F6bG9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A27279AB-E752-48D6-90F0-4DEB40BB185F}"/>
+    <hyperlink ref="AL261" r:id="rId120" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLYkZaVVZsWlZiRkpQVkRKV2MxWllaRlZOUmtwNVZHdFZOVlpYUmpaU2F6bFRVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A1E2B712-2AE5-4763-9710-D868EA63C98E}"/>
+    <hyperlink ref="AL263" r:id="rId121" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLYkZaVWJGWlZiRkpQVkRKV2MxWllaRlZOVmtwMVdrUkJlRTVzV2xWU2JFSlRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{B450DD8F-A365-485F-8E34-5C29DEB711B5}"/>
+    <hyperlink ref="AL266" r:id="rId122" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLYkdGNlZuaFZiRkpQVkRKV2MxWllhRlZXYkVwRFZGWlZOVkpXU2xWV2F6bHNZa1ZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{11ADDDFA-406F-459A-9505-70CE6AC22454}"/>
+    <hyperlink ref="AL268" r:id="rId123" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLYkdGNmJFWlZiRkpQVkRKV2MxWllaRlZOVmtwWFdsVlZNVkpXVWxWV2F6Vm9ZWHBGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{80D1828A-0B50-4997-8055-16BA0C6A513F}"/>
+    <hyperlink ref="AL271" r:id="rId124" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGxKVVJsWlZiRkpQVkRKV2MxWllhRlZXVmtwWFdrUkJOVlpXYTNwaVJUVlhVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{540F6133-B96B-4813-9995-CD0337C6FCFE}"/>
+    <hyperlink ref="AL275" r:id="rId125" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGxKVVZuaFZiRkpQVkRKV2MxWllhRlZXVmtwTFZHeFZlRlpXVGxsalJUVlRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{7E068EB1-738F-4A62-98E3-4703B233F7B8}"/>
+    <hyperlink ref="AL277" r:id="rId126" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGxKVWJFWlZiRkpQVkRKV2MxWllhRlZXVmtweFZGWlZlRlpXY0RaVWF6VnNZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{D2043630-36A6-4F8B-857B-531277FE3B5E}"/>
+    <hyperlink ref="AL278" r:id="rId127" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGxKVWJGWlZiRkpQVkRKV2MxWllaRlZOUmtwUFZGVlZNVTVzVWxWUmF6Vm9Za1paZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{26AAB86F-EBC1-443A-B2EA-B02BF6FE4864}"/>
+    <hyperlink ref="AL281" r:id="rId128" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGxaVVJUSlZiRkpQVkRKV2MxWllaRlZOUmtwRFZGUkJNVTV0UmpaV2F6bFRVakEwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{B5F33F2D-B1F8-4818-B1B8-0F31395BF874}"/>
+    <hyperlink ref="AL286" r:id="rId129" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGxaVWJFWlZiRkpQVkRKV2MxWllhRlZXVmtwNVdsVlZlRTVzWkZWV2F6Vm9ZbGRSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{FCA12D81-7B1A-4E44-895D-2376CB66880F}"/>
+    <hyperlink ref="AL287" r:id="rId130" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGxaVWJGWlZiRkpQVkRKV2MxWllhRlZXVmtwVFZHdFZlRkpXWkZsYVJrSlRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{AEEE0651-A0E8-488A-9E37-8BE6270D0B59}"/>
+    <hyperlink ref="AL290" r:id="rId131" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVG1GNlJUSlZiRkpQVkRKV2MxWllaRlZOUmtwSFdsVlZOVlpXUmxWUmF6VnNZbGhSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{98D6F3AB-D9DE-4D2A-81A7-C7EF62304F23}"/>
+    <hyperlink ref="AL291" r:id="rId132" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVG1GNlZrWlZiRkpQVkRKV2MxWllaRlZOVmtwMVdsVlZlRlpXU2xWUmF6VlRVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{F6530679-96A2-4C39-9102-C96DAED6B99B}"/>
+    <hyperlink ref="AL292" r:id="rId133" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVG1GNlZsWlZiRkpQVkRKV2MxWllaRlZOVmtwVFZGVlZlRlpXY0RaVmF6VlRVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{EA9E2AC2-C7FB-4605-B4F2-ABC589A238E1}"/>
+    <hyperlink ref="AL293" r:id="rId134" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVG1GNlZuaFZiRkpQVkRKV2MxWllaRlZOUmtwWFdsVlZNVlpXVmxWVmF6bG9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{E0C91A0D-D469-47FF-B8BA-CEC38AD66B81}"/>
+    <hyperlink ref="AL295" r:id="rId135" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVG1GNmJFWlZiRkpQVkRKV2MxWllaRlZOUmtwSFZGZHpOVlpXUmxsalJrSlhVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{2C382890-5866-440D-8AA6-717E6CA28233}"/>
+    <hyperlink ref="AL297" r:id="rId136" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGsxRVJrWlZiRkpQVkRKV2MxWllhRlZXVmtwUFdsVlZNVkpXYTNwalJUVnNZa1paZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{25B32894-5038-41BE-8BB6-FB180A35CAD2}"/>
+    <hyperlink ref="AL299" r:id="rId137" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGsxRVJuaFZiRkpQVkRKV2MxWllhRlZXVmtwWFZGVlZNVTV0UlhwaVJUbFRVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{9727FD14-6349-4D40-A788-6F082E527FDB}"/>
+    <hyperlink ref="AL300" r:id="rId138" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGsxRVJUSlZiRkpQVkRKV2MxWllaRlZOVmtwWFdsZHpNVlpXYTNwalJrSlhVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{79BD4801-4D4C-4A50-8C6C-3F44735FDF96}"/>
+    <hyperlink ref="AL302" r:id="rId139" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGsxRVZuaFZiRkpQVkRKV2MxWllaRlZOUmtwWFdrUkJNVkpYUmpaU2F6VlRVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{810C46C9-9FFB-40F0-B2F3-8252D35FAFAF}"/>
+    <hyperlink ref="AL304" r:id="rId140" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGsxRWJFWlZiRkpQVkRKV2MxWllaRlZOVmtwUFdsZHplRkpXYjNwYVJUbHNZbGRSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{1974B929-12D3-42DE-A908-E4B3C2D5B511}"/>
+    <hyperlink ref="AL305" r:id="rId141" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVGsxRWJGWlZiRkpQVkRKV2MxWllaRlZOVmtwRFdrUkJlRlpXYjNwYVJUVlRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{EBA376E0-D8C2-4B66-B940-8E00E43D8D8F}"/>
+    <hyperlink ref="AL306" r:id="rId142" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFKVVJrWlZiRkpQVkRKV2MxWllaRlZOVmtwWFZHdFZlRlpXV2xsalJUbG9ZbGhSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{AE51CC78-7661-4CA2-9E06-908C737F61DF}"/>
+    <hyperlink ref="AL307" r:id="rId143" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFKVVJsWlZiRkpQVkRKV2MxWllaRlZOVmtwRFZHeFZOVlpXVGxWU2F6bG9ZbGRSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{B8DD8597-0D22-4465-9B3F-A896759AF1D7}"/>
+    <hyperlink ref="AL308" r:id="rId144" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFKVVJuaFZiRkpQVkRKV2MxWllhRlZXVmtwWFZHdFZNVkpXU2xsYVJUbG9ZbGRSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{07A7B040-0B0A-4C0B-A0CF-F1503EA7B067}"/>
+    <hyperlink ref="AL309" r:id="rId145" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFKVVJUSlZiRkpQVkRKV2MxWllaRlZOVmtwSFZHdFZlRlpXUmxsaFJUbFRVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{698FC469-61DA-4FAB-A05D-B6949F5FFD36}"/>
+    <hyperlink ref="AL312" r:id="rId146" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFKVVZuaFZiRkpQVkRKV2MxWllaRlZOVmtwUFdsVlZlR05XVmxsaVJrSlhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{2AA2DE72-89A0-4D64-A355-F73B99B63C48}"/>
+    <hyperlink ref="AL313" r:id="rId147" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFKVVZUSlZiRkpQVkRKV2MxWllhRlZXVmtweFdsWlZNVkpXYkRaVWJFSlRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{92F0137E-85FA-425F-B056-2224B7A649D9}"/>
+    <hyperlink ref="AL320" r:id="rId148" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFaVVZrWlZiRkpQVkRKV2MxWllaRlZpYmtKNVZGWlZlRTVzV2xWU2F6bG9ZVEJaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{5B6FE16F-7BC8-46DF-A0F4-7B3AAA6CDCAC}"/>
+    <hyperlink ref="AL322" r:id="rId149" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFaVVZuaFZiRkpQVkRKV2MxWllhRlZXVmtwSFdsWlZlRlpXV2xWVmF6Vm9Za1ZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{F8F766FD-5899-4A59-971E-C59A190D0580}"/>
+    <hyperlink ref="AL323" r:id="rId150" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFaVVZUSlZiRkpQVkRKV2MxWllaRlZOUmtwaFdsZHplR05YUmpaVmJFSlhVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{73B0F1BB-7EFD-488A-94C3-C0DB360DAF69}"/>
+    <hyperlink ref="AL325" r:id="rId151" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFpLVDFaVWJGWlZiRkpQVkRKV2MxWllaRlZOUmtweFdsWlZlRlpXYkRaVGF6VnNZa1ZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{F5E0910A-A5F8-4C3E-9336-C468BB5CFDA2}"/>
+    <hyperlink ref="AL330" r:id="rId152" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYTAxRVZrWlZiRkpQVkRKV2MxWllaRlZOVmtwVFZGWlZNV05YUlhwaFJUVlRVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{84162CD3-F0F0-448D-8E2A-59F08BAC8D0E}"/>
+    <hyperlink ref="AL332" r:id="rId153" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYTAxRVZuaFZiRkpQVkRKV2MxWllaRlZOVmtwMVZGZHplRTVzVWxWU2JFSlhVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{57298DF6-8040-4A20-A7FE-F52E120199EA}"/>
+    <hyperlink ref="AL334" r:id="rId154" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYTAxRWJFWlZiRkpQVkRKV2MxWllaRlZOVmtwNVdsVlZNVTVzYTNwalJUbFRVak5SZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{518EF8E1-2D3F-4444-A28F-11DC4C997600}"/>
+    <hyperlink ref="AL337" r:id="rId155" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkZKVVJuaFZiRkpQVkRKV2MxWllhRlZXVmtweFZGVlZNVTVzU2xWVmJFSlhVak5SZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{63E1AC5E-9130-431A-B312-718788DA0AC8}"/>
+    <hyperlink ref="AL338" r:id="rId156" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkZKVVJUSlZiRkpQVkRKV2MxWllaRlZOVmtweFZGVlZNVlpXU2xWVWF6bG9Za1paZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{8B7743FB-C3F4-4067-8D33-B69DBC0934B8}"/>
+    <hyperlink ref="AL342" r:id="rId157" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkZKVVZUSlZiRkpQVkRKV2MxWllhRlZXVmtweFZHdFZlRlpXYTNwaFJUVnNZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{5E53CC60-DC80-46FA-A95B-F7FA84954816}"/>
+    <hyperlink ref="AL343" r:id="rId158" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkZKVWJFWlZiRkpQVkRKV2MxWllhRlZXVmtwVFdsWlZlRkpXUmxWUmF6bFhVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{FFD38858-E0FA-4E9F-8E93-0FFDEB990640}"/>
+    <hyperlink ref="AL344" r:id="rId159" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkZKVWJGWlZiRkpQVkRKV2MxWllhRlZXVmtweFZGWlZlRlpXYjNwYVJUbG9ZWHBGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{67818977-10DA-45CA-A595-37CF8D592624}"/>
+    <hyperlink ref="AL346" r:id="rId160" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkZaVVJuaFZiRkpQVkRKV2MxWllhRlZXVmtwUFZGVlZlRTVzV2xWV2F6bG9Za1ZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{5B7407A6-8C36-4EE0-9C33-766B6AB18F92}"/>
+    <hyperlink ref="AL354" r:id="rId161" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkdGNlJuaFZiRkpQVkRKV2MxWllaRlZOUmtwVFZGUkJlRkpXVGxsaFJrSlRVakpSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{423BBF50-FB18-4225-B4E6-059FBCF0347E}"/>
+    <hyperlink ref="AL355" r:id="rId162" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkdGNlJUSlZiRkpQVkRKV2MxWllaRlZOVmtwSFZHdFZOVkpXY0RaU2F6bHNZWHBGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{15F154E2-AA71-44D5-9DF8-FAD179E52FBD}"/>
+    <hyperlink ref="AL356" r:id="rId163" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkdGNlZrWlZiRkpQVkRKV2MxWllhRlZXVmtwUFdsVlZNVlpXVmxWU2JFSlRVbXhaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{F80F4EEF-DEB4-435F-8082-EB71FB7574C4}"/>
+    <hyperlink ref="AL357" r:id="rId164" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkdGNlZsWlZiRkpQVkRKV2MxWllaRlZOUmtwMVdsVlZNVlpXV2xWVWF6Vm9Za1paZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{61558F19-DFB6-4582-ACF4-D2F284DE006A}"/>
+    <hyperlink ref="AL358" r:id="rId165" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphYkdGNlZuaFZiRkpQVkRKV2MxWllhRlZXVmtwWFZGZHpNVkpXVWxWVmF6bG9ZVEZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{2B05624F-D8DF-40E6-AFBC-5448837F5DB0}"/>
+    <hyperlink ref="AL364" r:id="rId166" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxKVVJUSlZiRkpQVkRKV2MxWllaRlZOVmtwWFZHdFZNV05XV2xsYVJrSlRVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{8A7BD8CC-C6B7-4DE0-A41D-46C00C04AA87}"/>
+    <hyperlink ref="AL365" r:id="rId167" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxKVVZuaFZiRkpQVkRKV2MxWllaRlZOVmtwWFdsWlZlRTVzVWxWVmJFSlRVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{D1E825CA-8E5F-4F24-8390-C3E12AE44896}"/>
+    <hyperlink ref="AL366" r:id="rId168" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxKVVZUSlZiRkpQVkRKV2MxWllaRlZOVmtwMVZGWlZlRlpXY0RaVmF6VnNZa2QzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{06CB37E2-777F-448A-9BB3-F1771C0AF70A}"/>
+    <hyperlink ref="AL367" r:id="rId169" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxKVWJFWlZiRkpQVkRKV2MxWllhRlZXVmtwaFZHeFZNV05XVmxsYVJUVm9ZVEZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{0B806395-72D1-4159-91C8-33D8D69B8FC6}"/>
+    <hyperlink ref="AL369" r:id="rId170" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxaVVJsWlZiRkpQVkRKV2MxWllaRlZpYmtKMVZGUkJlRTVzV2xWUmF6bHNZa1paZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{DF9778AC-1C83-402F-981C-4687227993F0}"/>
+    <hyperlink ref="AL370" r:id="rId171" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxaVVJUSlZiRkpQVkRKV2MxWllaRlZOUmtwNVdrUkJNVlpXWkZWUmF6VlhVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{4B055990-4079-4232-9EB6-8E7409481BCD}"/>
+    <hyperlink ref="AL372" r:id="rId172" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxaVVZuaFZiRkpQVkRKV2MxWllaRlZpYmtKNVZGVlZNVlpYUmpaU2F6VnNZWHBGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{64FC1BA3-9960-46AA-BE40-E9C8392AFFCB}"/>
+    <hyperlink ref="AL373" r:id="rId173" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxaVVZUSlZiRkpQVkRKV2MxWllaRlZOUmtwRFZGZHplR05XYkRaVmF6bFhVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{42E89AE7-6B9C-4753-A277-120E6386DE8F}"/>
+    <hyperlink ref="AL374" r:id="rId174" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxaVWJFWlZiRkpQVkRKV2MxWllaRlZOUmtwRFdsVlZlRkpXWkZsYVJUbFRVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A816B7CC-B0A9-4255-BC71-3F4F99DBC8AA}"/>
+    <hyperlink ref="AL375" r:id="rId175" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVG1GNlJsWlZiRkpQVkRKV2MxWllaRlZOUmtwTFZGUkJNV05XVGxWVGF6VlRVbFZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{B7068F7E-35E8-45BE-8C4E-87B97EA20ED5}"/>
+    <hyperlink ref="AL376" r:id="rId176" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVG1GNlJuaFZiRkpQVkRKV2MxWllaRlZOVmtwUFZGUkJOVlpXV2xWUmF6bFhVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{8AE2B8F8-8AD8-4834-8626-D19BD8DDC6D7}"/>
+    <hyperlink ref="AL377" r:id="rId177" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVG1GNlJUSlZiRkpQVkRKV2MxWllaRlZOUmtwUFZGVlZOVkpXVmxWVmJFSlhVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{61095A65-66AA-4B96-A9A1-06072BB571FD}"/>
+    <hyperlink ref="AL378" r:id="rId178" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVG1GNlZrWlZiRkpQVkRKV2MxWllaRlZOVmtwTFZHdFZNV05XWkZWV2F6bHNZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{0D39699B-963C-4820-B390-7C9F15A09D00}"/>
+    <hyperlink ref="AL380" r:id="rId179" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVG1GNlZuaFZiRkpQVkRKV2MxWllaRlZOVmtwTFdsZHpOVkpXVWxsaFJUVlRVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A0526406-AAF0-4071-8E02-2083C911B390}"/>
+    <hyperlink ref="AL381" r:id="rId180" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVG1GNlZUSlZiRkpQVkRKV2MxWllaRlZOVmtwTFdsVlZNVlpXVGxWVmF6bFhVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A4F41422-E40B-405D-9CFD-EE6D798BE879}"/>
+    <hyperlink ref="AL383" r:id="rId181" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGsxRVJUSlZiRkpQVkRKV2MxWllaRlZOVmtwTFZGWlZlRTVzVGxWV2F6bG9ZWHBGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{D0C67FBB-C9DB-4173-87A9-97097FE17706}"/>
+    <hyperlink ref="AL384" r:id="rId182" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGsxRVZrWlZiRkpQVkRKV2MxWllhRlZXVmtwaFZGZHpNVTVzU2xWV2F6bFhVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{8C02CFEB-02D8-41EC-A515-993A9A178E54}"/>
+    <hyperlink ref="AL385" r:id="rId183" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGsxRVZsWlZiRkpQVkRKV2MxWllhRlZXVmtwWFZHdFZNVkpXY0RaV2F6VlhVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{843628D7-BA73-43C4-8720-D71676E75F77}"/>
+    <hyperlink ref="AL386" r:id="rId184" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGsxRVZuaFZiRkpQVkRKV2MxWllaRlZOVmtwVFdsWlZlRTV0UlhwaFJUVnNZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{4334B7C1-7D57-4317-8C00-6E42CC58FF95}"/>
+    <hyperlink ref="AL387" r:id="rId185" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGsxRVZUSlZiRkpQVkRKV2MxWllaRlZOVmtwVFZGZHpNVTVzV2xWVWJFSlRVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{1A7126A5-BAB1-48A9-BBFD-B0C727FA913B}"/>
+    <hyperlink ref="AL388" r:id="rId186" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGsxRWJFWlZiRkpQVkRKV2MxWllhRlZXVmtweFdsZHpOVlpXVGxWVmF6bFRVbTEzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{C5181940-1A5B-4D5D-94A4-6130583BFDAF}"/>
+    <hyperlink ref="AL391" r:id="rId187" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVDFKVVZrWlZiRkpQVkRKV2MxWllhRlZXYkVwRFdsWlZlRTVzVmxWVWF6VlhVbFpaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{EF0C3738-0571-4BBB-91C7-8B7E671E97A5}"/>
+    <hyperlink ref="AL395" r:id="rId188" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVDFaVVJrWlZiRkpQVkRKV2MxWllaRlZOVmtwUFZHdFZOVlpXU2xsaVJUbG9Za1ZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{627425C4-DAF8-407B-AFA7-5964657463DC}"/>
+    <hyperlink ref="AL396" r:id="rId189" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVDFaVVJsWlZiRkpQVkRKV2MxWllaRlZOVmtwTFZGWlZlR05XVWxsaVJUbHNZbGRSZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{28EA5126-180F-48C1-9CDA-F9DFF35C0614}"/>
+    <hyperlink ref="AL425" r:id="rId190" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzVLYkZKVVJrWlZiRkpQVkRKV2MxWllaRlZOUmtwaFdsWlZlR05XVWxsaVJUbFhVbXRaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{A12F385C-F600-4B1E-82E9-1FF454B95162}"/>
+    <hyperlink ref="AL436" r:id="rId191" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSllZMFphVGxKVVZrWlZiRkpQVkRKV2MxWllaRlZOVmtwSFZGUkJNV05XYTNwaVJUbG9Za1ZaZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{4B4D7322-3C51-42B9-B3C6-B98D0E7D3DEB}"/>
+    <hyperlink ref="AL438" r:id="rId192" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlhWVzAxVDFKVVZUSlZiRkpQVkRKV2MxWllaRlZOVmtwTFdsWlZNVTVzVWxWV2F6Vm9ZVEozZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{AD6F295A-BB74-455B-B728-6581E10081B5}"/>
+    <hyperlink ref="AL442" r:id="rId193" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlpZMFZLVDFKVVZUSlZiRkpQVkRKV2MxWllaRlZOVmtwMVZHdFZlRTV0UmpaVmF6VnNZbFUwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{FF7D5119-F1FA-427A-A0FB-69BA836C8F88}"/>
+    <hyperlink ref="AL445" r:id="rId194" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlpZMFZLVDFaVVJrWlZiRkpQVkRKV2MxWllaRlZOVmtwWFZGWlZNVTVzVWxWVmF6VlRVbFJGZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{B9136A3F-CB21-4307-AB52-C664B9A87FC7}"/>
+    <hyperlink ref="AL449" r:id="rId195" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlpZMFZLVDFaVVZrWlZiRkpQVkRKV2MxWllaRlZOVmtwTFdsWlZlR05XUmxWVWF6VlRVakEwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{DF958B4F-AC7F-4CF9-903F-28A306A00A92}"/>
+    <hyperlink ref="AL452" r:id="rId196" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSlpZMFZLVDFaVVZUSlZiRkpQVkRKV2MxWllhRlZXVmtwSFZHdFZlRTVzU2xWV2F6VlhVakEwZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{DD6E74FA-E1DE-4AE1-A5B8-2118E3A04395}"/>
+    <hyperlink ref="AL499" r:id="rId197" display="https://eic.godoworks.com/v2_0/getImagews.php?t=1775528592&amp;id=Vmxkd1ExVXhaRWRoUkZwVFZrVTFUMVpyWkU1a01WSnlWV3MxYkdGNlJrWlZiRkpQVkRKV2MxWllaRlZOUmtwNVZGVlZlR05XYjNwalJUbFhVbGQzZUZkV1l6RlJNa3B1VUZRd1BRPT0rUA==&amp;cuenta=705" xr:uid="{F9605E40-235F-4D7C-83AE-8EAD6BC59669}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>